<commit_message>
Update NBA sim outputs (2026-04-03)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_matchup_probs.xlsx
+++ b/nba/public/data/nba_matchup_probs.xlsx
@@ -843,19 +843,19 @@
         <v>0.7216</v>
       </c>
       <c r="H8" t="n">
-        <v>0.5381</v>
+        <v>0.5417</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6298</v>
+        <v>0.6316000000000001</v>
       </c>
       <c r="J8" t="n">
         <v>0.2784</v>
       </c>
       <c r="K8" t="n">
-        <v>0.4619</v>
+        <v>0.4583</v>
       </c>
       <c r="L8" t="n">
-        <v>0.3702</v>
+        <v>0.3684</v>
       </c>
       <c r="M8" t="n">
         <v>164</v>
@@ -1221,19 +1221,19 @@
         <v>0.8678</v>
       </c>
       <c r="H15" t="n">
-        <v>0.7642</v>
+        <v>0.7739</v>
       </c>
       <c r="I15" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.8208</v>
       </c>
       <c r="J15" t="n">
         <v>0.1322</v>
       </c>
       <c r="K15" t="n">
-        <v>0.2358</v>
+        <v>0.2261</v>
       </c>
       <c r="L15" t="n">
-        <v>0.184</v>
+        <v>0.1792</v>
       </c>
       <c r="M15" t="n">
         <v>164</v>
@@ -1380,22 +1380,22 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>0.8148</v>
+        <v>0.8126</v>
       </c>
       <c r="H18" t="n">
-        <v>0.6931</v>
+        <v>0.6911</v>
       </c>
       <c r="I18" t="n">
-        <v>0.754</v>
+        <v>0.7518</v>
       </c>
       <c r="J18" t="n">
-        <v>0.1852</v>
+        <v>0.1874</v>
       </c>
       <c r="K18" t="n">
-        <v>0.3069</v>
+        <v>0.3089</v>
       </c>
       <c r="L18" t="n">
-        <v>0.246</v>
+        <v>0.2482</v>
       </c>
       <c r="M18" t="n">
         <v>164</v>
@@ -2028,22 +2028,22 @@
         </is>
       </c>
       <c r="G30" t="n">
-        <v>0.5456</v>
+        <v>0.5218</v>
       </c>
       <c r="H30" t="n">
-        <v>0.407</v>
+        <v>0.4053</v>
       </c>
       <c r="I30" t="n">
-        <v>0.4763</v>
+        <v>0.4636</v>
       </c>
       <c r="J30" t="n">
-        <v>0.4544</v>
+        <v>0.4782</v>
       </c>
       <c r="K30" t="n">
-        <v>0.593</v>
+        <v>0.5947</v>
       </c>
       <c r="L30" t="n">
-        <v>0.5237000000000001</v>
+        <v>0.5364</v>
       </c>
       <c r="M30" t="n">
         <v>164</v>
@@ -2193,19 +2193,19 @@
         <v>0.8582</v>
       </c>
       <c r="H33" t="n">
-        <v>0.7382</v>
+        <v>0.74</v>
       </c>
       <c r="I33" t="n">
-        <v>0.7982</v>
+        <v>0.7991</v>
       </c>
       <c r="J33" t="n">
         <v>0.1418</v>
       </c>
       <c r="K33" t="n">
-        <v>0.2618</v>
+        <v>0.26</v>
       </c>
       <c r="L33" t="n">
-        <v>0.2018</v>
+        <v>0.2009</v>
       </c>
       <c r="M33" t="n">
         <v>164</v>
@@ -2892,22 +2892,22 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>0.8623</v>
+        <v>0.8594000000000001</v>
       </c>
       <c r="H46" t="n">
-        <v>0.7581</v>
+        <v>0.7529</v>
       </c>
       <c r="I46" t="n">
-        <v>0.8102</v>
+        <v>0.8062</v>
       </c>
       <c r="J46" t="n">
-        <v>0.1377</v>
+        <v>0.1406</v>
       </c>
       <c r="K46" t="n">
-        <v>0.2419</v>
+        <v>0.2471</v>
       </c>
       <c r="L46" t="n">
-        <v>0.1898</v>
+        <v>0.1938</v>
       </c>
       <c r="M46" t="n">
         <v>164</v>
@@ -3540,22 +3540,22 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>0.6906</v>
+        <v>0.6728</v>
       </c>
       <c r="H58" t="n">
-        <v>0.5284</v>
+        <v>0.5187</v>
       </c>
       <c r="I58" t="n">
-        <v>0.6095</v>
+        <v>0.5958</v>
       </c>
       <c r="J58" t="n">
-        <v>0.3094</v>
+        <v>0.3272</v>
       </c>
       <c r="K58" t="n">
-        <v>0.4716</v>
+        <v>0.4813</v>
       </c>
       <c r="L58" t="n">
-        <v>0.3905</v>
+        <v>0.4042</v>
       </c>
       <c r="M58" t="n">
         <v>164</v>
@@ -4350,22 +4350,22 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>0.8442</v>
+        <v>0.8366</v>
       </c>
       <c r="H73" t="n">
         <v>0.7727000000000001</v>
       </c>
       <c r="I73" t="n">
-        <v>0.8084</v>
+        <v>0.8047</v>
       </c>
       <c r="J73" t="n">
-        <v>0.1558</v>
+        <v>0.1634</v>
       </c>
       <c r="K73" t="n">
         <v>0.2273</v>
       </c>
       <c r="L73" t="n">
-        <v>0.1916</v>
+        <v>0.1953</v>
       </c>
       <c r="M73" t="n">
         <v>164</v>
@@ -4404,22 +4404,22 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>0.7541</v>
+        <v>0.7565</v>
       </c>
       <c r="H74" t="n">
         <v>0.6133</v>
       </c>
       <c r="I74" t="n">
-        <v>0.6837</v>
+        <v>0.6849</v>
       </c>
       <c r="J74" t="n">
-        <v>0.2459</v>
+        <v>0.2435</v>
       </c>
       <c r="K74" t="n">
         <v>0.3867</v>
       </c>
       <c r="L74" t="n">
-        <v>0.3163</v>
+        <v>0.3151</v>
       </c>
       <c r="M74" t="n">
         <v>164</v>
@@ -4458,22 +4458,22 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>0.7549</v>
+        <v>0.7571</v>
       </c>
       <c r="H75" t="n">
         <v>0.6009</v>
       </c>
       <c r="I75" t="n">
-        <v>0.6778999999999999</v>
+        <v>0.679</v>
       </c>
       <c r="J75" t="n">
-        <v>0.2451</v>
+        <v>0.2429</v>
       </c>
       <c r="K75" t="n">
         <v>0.3991</v>
       </c>
       <c r="L75" t="n">
-        <v>0.3221</v>
+        <v>0.321</v>
       </c>
       <c r="M75" t="n">
         <v>164</v>
@@ -4998,22 +4998,22 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>0.6502</v>
+        <v>0.6398</v>
       </c>
       <c r="H85" t="n">
-        <v>0.5044999999999999</v>
+        <v>0.4883</v>
       </c>
       <c r="I85" t="n">
-        <v>0.5774</v>
+        <v>0.5641</v>
       </c>
       <c r="J85" t="n">
-        <v>0.3498</v>
+        <v>0.3602</v>
       </c>
       <c r="K85" t="n">
-        <v>0.4955</v>
+        <v>0.5117</v>
       </c>
       <c r="L85" t="n">
-        <v>0.4226</v>
+        <v>0.4359</v>
       </c>
       <c r="M85" t="n">
         <v>164</v>
@@ -5160,22 +5160,22 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>0.2764</v>
+        <v>0.2717</v>
       </c>
       <c r="H88" t="n">
         <v>0.1604</v>
       </c>
       <c r="I88" t="n">
-        <v>0.2184</v>
+        <v>0.216</v>
       </c>
       <c r="J88" t="n">
-        <v>0.7236</v>
+        <v>0.7282999999999999</v>
       </c>
       <c r="K88" t="n">
         <v>0.8396</v>
       </c>
       <c r="L88" t="n">
-        <v>0.7816</v>
+        <v>0.784</v>
       </c>
       <c r="M88" t="n">
         <v>164</v>
@@ -5754,22 +5754,22 @@
         </is>
       </c>
       <c r="G99" t="n">
-        <v>0.6327</v>
+        <v>0.628</v>
       </c>
       <c r="H99" t="n">
-        <v>0.495</v>
+        <v>0.4944</v>
       </c>
       <c r="I99" t="n">
-        <v>0.5638</v>
+        <v>0.5612</v>
       </c>
       <c r="J99" t="n">
-        <v>0.3673</v>
+        <v>0.372</v>
       </c>
       <c r="K99" t="n">
-        <v>0.505</v>
+        <v>0.5056</v>
       </c>
       <c r="L99" t="n">
-        <v>0.4362</v>
+        <v>0.4388</v>
       </c>
       <c r="M99" t="n">
         <v>164</v>
@@ -6402,22 +6402,22 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>0.3517</v>
+        <v>0.3441</v>
       </c>
       <c r="H111" t="n">
-        <v>0.2045</v>
+        <v>0.2</v>
       </c>
       <c r="I111" t="n">
-        <v>0.2781</v>
+        <v>0.272</v>
       </c>
       <c r="J111" t="n">
-        <v>0.6483</v>
+        <v>0.6559</v>
       </c>
       <c r="K111" t="n">
-        <v>0.7955</v>
+        <v>0.8</v>
       </c>
       <c r="L111" t="n">
-        <v>0.7219</v>
+        <v>0.728</v>
       </c>
       <c r="M111" t="n">
         <v>164</v>
@@ -6729,19 +6729,19 @@
         <v>0.3749</v>
       </c>
       <c r="H117" t="n">
-        <v>0.2191</v>
+        <v>0.2203</v>
       </c>
       <c r="I117" t="n">
-        <v>0.297</v>
+        <v>0.2976</v>
       </c>
       <c r="J117" t="n">
         <v>0.6251</v>
       </c>
       <c r="K117" t="n">
-        <v>0.7809</v>
+        <v>0.7796999999999999</v>
       </c>
       <c r="L117" t="n">
-        <v>0.703</v>
+        <v>0.7024</v>
       </c>
       <c r="M117" t="n">
         <v>164</v>
@@ -7104,22 +7104,22 @@
         </is>
       </c>
       <c r="G124" t="n">
-        <v>0.6226</v>
+        <v>0.6029</v>
       </c>
       <c r="H124" t="n">
-        <v>0.5004999999999999</v>
+        <v>0.4985</v>
       </c>
       <c r="I124" t="n">
-        <v>0.5616</v>
+        <v>0.5507</v>
       </c>
       <c r="J124" t="n">
-        <v>0.3774</v>
+        <v>0.3971</v>
       </c>
       <c r="K124" t="n">
-        <v>0.4995</v>
+        <v>0.5014999999999999</v>
       </c>
       <c r="L124" t="n">
-        <v>0.4384</v>
+        <v>0.4493</v>
       </c>
       <c r="M124" t="n">
         <v>164</v>
@@ -7752,22 +7752,22 @@
         </is>
       </c>
       <c r="G136" t="n">
-        <v>0.3529</v>
+        <v>0.3379</v>
       </c>
       <c r="H136" t="n">
-        <v>0.2004</v>
+        <v>0.1836</v>
       </c>
       <c r="I136" t="n">
-        <v>0.2766</v>
+        <v>0.2608</v>
       </c>
       <c r="J136" t="n">
-        <v>0.6471</v>
+        <v>0.6621</v>
       </c>
       <c r="K136" t="n">
-        <v>0.7996</v>
+        <v>0.8164</v>
       </c>
       <c r="L136" t="n">
-        <v>0.7234</v>
+        <v>0.7392</v>
       </c>
       <c r="M136" t="n">
         <v>164</v>
@@ -8400,22 +8400,22 @@
         </is>
       </c>
       <c r="G148" t="n">
-        <v>0.5383</v>
+        <v>0.5357</v>
       </c>
       <c r="H148" t="n">
-        <v>0.4514</v>
+        <v>0.4429</v>
       </c>
       <c r="I148" t="n">
-        <v>0.4948</v>
+        <v>0.4893</v>
       </c>
       <c r="J148" t="n">
-        <v>0.4617</v>
+        <v>0.4643</v>
       </c>
       <c r="K148" t="n">
-        <v>0.5486</v>
+        <v>0.5571</v>
       </c>
       <c r="L148" t="n">
-        <v>0.5052</v>
+        <v>0.5107</v>
       </c>
       <c r="M148" t="n">
         <v>164</v>
@@ -8940,22 +8940,22 @@
         </is>
       </c>
       <c r="G158" t="n">
-        <v>0.6973</v>
+        <v>0.7019</v>
       </c>
       <c r="H158" t="n">
         <v>0.5595</v>
       </c>
       <c r="I158" t="n">
-        <v>0.6284</v>
+        <v>0.6307</v>
       </c>
       <c r="J158" t="n">
-        <v>0.3027</v>
+        <v>0.2981</v>
       </c>
       <c r="K158" t="n">
         <v>0.4405</v>
       </c>
       <c r="L158" t="n">
-        <v>0.3716</v>
+        <v>0.3693</v>
       </c>
       <c r="M158" t="n">
         <v>164</v>
@@ -9048,22 +9048,22 @@
         </is>
       </c>
       <c r="G160" t="n">
-        <v>0.2932</v>
+        <v>0.2837</v>
       </c>
       <c r="H160" t="n">
-        <v>0.163</v>
+        <v>0.1549</v>
       </c>
       <c r="I160" t="n">
-        <v>0.2281</v>
+        <v>0.2193</v>
       </c>
       <c r="J160" t="n">
-        <v>0.7068</v>
+        <v>0.7163</v>
       </c>
       <c r="K160" t="n">
-        <v>0.837</v>
+        <v>0.8451</v>
       </c>
       <c r="L160" t="n">
-        <v>0.7719</v>
+        <v>0.7806999999999999</v>
       </c>
       <c r="M160" t="n">
         <v>164</v>
@@ -9642,22 +9642,22 @@
         </is>
       </c>
       <c r="G171" t="n">
-        <v>0.8518</v>
+        <v>0.8478</v>
       </c>
       <c r="H171" t="n">
-        <v>0.7474</v>
+        <v>0.7421</v>
       </c>
       <c r="I171" t="n">
-        <v>0.7996</v>
+        <v>0.795</v>
       </c>
       <c r="J171" t="n">
-        <v>0.1482</v>
+        <v>0.1522</v>
       </c>
       <c r="K171" t="n">
-        <v>0.2526</v>
+        <v>0.2579</v>
       </c>
       <c r="L171" t="n">
-        <v>0.2004</v>
+        <v>0.205</v>
       </c>
       <c r="M171" t="n">
         <v>164</v>
@@ -10236,22 +10236,22 @@
         </is>
       </c>
       <c r="G182" t="n">
-        <v>0.6566</v>
+        <v>0.6607</v>
       </c>
       <c r="H182" t="n">
         <v>0.4997</v>
       </c>
       <c r="I182" t="n">
-        <v>0.5780999999999999</v>
+        <v>0.5802</v>
       </c>
       <c r="J182" t="n">
-        <v>0.3434</v>
+        <v>0.3393</v>
       </c>
       <c r="K182" t="n">
         <v>0.5003</v>
       </c>
       <c r="L182" t="n">
-        <v>0.4219</v>
+        <v>0.4198</v>
       </c>
       <c r="M182" t="n">
         <v>164</v>
@@ -10290,22 +10290,22 @@
         </is>
       </c>
       <c r="G183" t="n">
-        <v>0.6593</v>
+        <v>0.649</v>
       </c>
       <c r="H183" t="n">
-        <v>0.5139</v>
+        <v>0.4952</v>
       </c>
       <c r="I183" t="n">
-        <v>0.5866</v>
+        <v>0.5721000000000001</v>
       </c>
       <c r="J183" t="n">
-        <v>0.3407</v>
+        <v>0.351</v>
       </c>
       <c r="K183" t="n">
-        <v>0.4861</v>
+        <v>0.5048</v>
       </c>
       <c r="L183" t="n">
-        <v>0.4134</v>
+        <v>0.4279</v>
       </c>
       <c r="M183" t="n">
         <v>164</v>
@@ -10830,22 +10830,22 @@
         </is>
       </c>
       <c r="G193" t="n">
-        <v>0.7344000000000001</v>
+        <v>0.7194</v>
       </c>
       <c r="H193" t="n">
-        <v>0.5541</v>
+        <v>0.5537</v>
       </c>
       <c r="I193" t="n">
-        <v>0.6442</v>
+        <v>0.6365</v>
       </c>
       <c r="J193" t="n">
-        <v>0.2656</v>
+        <v>0.2806</v>
       </c>
       <c r="K193" t="n">
-        <v>0.4459</v>
+        <v>0.4463</v>
       </c>
       <c r="L193" t="n">
-        <v>0.3558</v>
+        <v>0.3635</v>
       </c>
       <c r="M193" t="n">
         <v>164</v>
@@ -11478,22 +11478,22 @@
         </is>
       </c>
       <c r="G205" t="n">
-        <v>0.4158</v>
+        <v>0.4017</v>
       </c>
       <c r="H205" t="n">
-        <v>0.2463</v>
+        <v>0.2364</v>
       </c>
       <c r="I205" t="n">
-        <v>0.331</v>
+        <v>0.319</v>
       </c>
       <c r="J205" t="n">
-        <v>0.5842000000000001</v>
+        <v>0.5983000000000001</v>
       </c>
       <c r="K205" t="n">
-        <v>0.7537</v>
+        <v>0.7635999999999999</v>
       </c>
       <c r="L205" t="n">
-        <v>0.669</v>
+        <v>0.681</v>
       </c>
       <c r="M205" t="n">
         <v>164</v>
@@ -11964,22 +11964,22 @@
         </is>
       </c>
       <c r="G214" t="n">
-        <v>0.8256</v>
+        <v>0.8202</v>
       </c>
       <c r="H214" t="n">
-        <v>0.7187</v>
+        <v>0.7106</v>
       </c>
       <c r="I214" t="n">
-        <v>0.7722</v>
+        <v>0.7654</v>
       </c>
       <c r="J214" t="n">
-        <v>0.1744</v>
+        <v>0.1798</v>
       </c>
       <c r="K214" t="n">
-        <v>0.2813</v>
+        <v>0.2894</v>
       </c>
       <c r="L214" t="n">
-        <v>0.2278</v>
+        <v>0.2346</v>
       </c>
       <c r="M214" t="n">
         <v>164</v>
@@ -12612,22 +12612,22 @@
         </is>
       </c>
       <c r="G226" t="n">
-        <v>0.5876</v>
+        <v>0.5669</v>
       </c>
       <c r="H226" t="n">
-        <v>0.4576</v>
+        <v>0.4527</v>
       </c>
       <c r="I226" t="n">
-        <v>0.5226</v>
+        <v>0.5098</v>
       </c>
       <c r="J226" t="n">
-        <v>0.4124</v>
+        <v>0.4331</v>
       </c>
       <c r="K226" t="n">
-        <v>0.5424</v>
+        <v>0.5473</v>
       </c>
       <c r="L226" t="n">
-        <v>0.4774</v>
+        <v>0.4902</v>
       </c>
       <c r="M226" t="n">
         <v>164</v>
@@ -13044,22 +13044,22 @@
         </is>
       </c>
       <c r="G234" t="n">
-        <v>0.8128</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H234" t="n">
-        <v>0.6944</v>
+        <v>0.6815</v>
       </c>
       <c r="I234" t="n">
-        <v>0.7536</v>
+        <v>0.7458</v>
       </c>
       <c r="J234" t="n">
-        <v>0.1872</v>
+        <v>0.19</v>
       </c>
       <c r="K234" t="n">
-        <v>0.3056</v>
+        <v>0.3185</v>
       </c>
       <c r="L234" t="n">
-        <v>0.2464</v>
+        <v>0.2542</v>
       </c>
       <c r="M234" t="n">
         <v>164</v>
@@ -13479,19 +13479,19 @@
         <v>0.8381</v>
       </c>
       <c r="H242" t="n">
-        <v>0.7088</v>
+        <v>0.7122000000000001</v>
       </c>
       <c r="I242" t="n">
-        <v>0.7734</v>
+        <v>0.7752</v>
       </c>
       <c r="J242" t="n">
         <v>0.1619</v>
       </c>
       <c r="K242" t="n">
-        <v>0.2912</v>
+        <v>0.2878</v>
       </c>
       <c r="L242" t="n">
-        <v>0.2266</v>
+        <v>0.2248</v>
       </c>
       <c r="M242" t="n">
         <v>164</v>
@@ -13692,22 +13692,22 @@
         </is>
       </c>
       <c r="G246" t="n">
-        <v>0.5007</v>
+        <v>0.4889</v>
       </c>
       <c r="H246" t="n">
-        <v>0.4137</v>
+        <v>0.4023</v>
       </c>
       <c r="I246" t="n">
-        <v>0.4572</v>
+        <v>0.4456</v>
       </c>
       <c r="J246" t="n">
-        <v>0.4993</v>
+        <v>0.5111</v>
       </c>
       <c r="K246" t="n">
-        <v>0.5863</v>
+        <v>0.5977</v>
       </c>
       <c r="L246" t="n">
-        <v>0.5427999999999999</v>
+        <v>0.5544</v>
       </c>
       <c r="M246" t="n">
         <v>164</v>
@@ -14070,22 +14070,22 @@
         </is>
       </c>
       <c r="G253" t="n">
-        <v>0.8114</v>
+        <v>0.8001</v>
       </c>
       <c r="H253" t="n">
-        <v>0.6961000000000001</v>
+        <v>0.6839</v>
       </c>
       <c r="I253" t="n">
-        <v>0.7538</v>
+        <v>0.742</v>
       </c>
       <c r="J253" t="n">
-        <v>0.1886</v>
+        <v>0.1999</v>
       </c>
       <c r="K253" t="n">
-        <v>0.3039</v>
+        <v>0.3161</v>
       </c>
       <c r="L253" t="n">
-        <v>0.2462</v>
+        <v>0.258</v>
       </c>
       <c r="M253" t="n">
         <v>164</v>
@@ -14286,22 +14286,22 @@
         </is>
       </c>
       <c r="G257" t="n">
-        <v>0.8431</v>
+        <v>0.8458</v>
       </c>
       <c r="H257" t="n">
         <v>0.735</v>
       </c>
       <c r="I257" t="n">
-        <v>0.789</v>
+        <v>0.7904</v>
       </c>
       <c r="J257" t="n">
-        <v>0.1569</v>
+        <v>0.1542</v>
       </c>
       <c r="K257" t="n">
         <v>0.265</v>
       </c>
       <c r="L257" t="n">
-        <v>0.211</v>
+        <v>0.2096</v>
       </c>
       <c r="M257" t="n">
         <v>164</v>
@@ -14397,19 +14397,19 @@
         <v>0.361</v>
       </c>
       <c r="H259" t="n">
-        <v>0.2354</v>
+        <v>0.2331</v>
       </c>
       <c r="I259" t="n">
-        <v>0.2982</v>
+        <v>0.297</v>
       </c>
       <c r="J259" t="n">
         <v>0.639</v>
       </c>
       <c r="K259" t="n">
-        <v>0.7645999999999999</v>
+        <v>0.7669</v>
       </c>
       <c r="L259" t="n">
-        <v>0.7018</v>
+        <v>0.703</v>
       </c>
       <c r="M259" t="n">
         <v>164</v>
@@ -14718,22 +14718,22 @@
         </is>
       </c>
       <c r="G265" t="n">
-        <v>0.4949</v>
+        <v>0.4729</v>
       </c>
       <c r="H265" t="n">
-        <v>0.4292</v>
+        <v>0.4214</v>
       </c>
       <c r="I265" t="n">
-        <v>0.462</v>
+        <v>0.4472</v>
       </c>
       <c r="J265" t="n">
-        <v>0.5051</v>
+        <v>0.5271</v>
       </c>
       <c r="K265" t="n">
-        <v>0.5708</v>
+        <v>0.5786</v>
       </c>
       <c r="L265" t="n">
-        <v>0.538</v>
+        <v>0.5528</v>
       </c>
       <c r="M265" t="n">
         <v>164</v>
@@ -15042,22 +15042,22 @@
         </is>
       </c>
       <c r="G271" t="n">
-        <v>0.7435</v>
+        <v>0.7316</v>
       </c>
       <c r="H271" t="n">
-        <v>0.5924</v>
+        <v>0.5878</v>
       </c>
       <c r="I271" t="n">
-        <v>0.668</v>
+        <v>0.6597</v>
       </c>
       <c r="J271" t="n">
-        <v>0.2565</v>
+        <v>0.2684</v>
       </c>
       <c r="K271" t="n">
-        <v>0.4076</v>
+        <v>0.4122</v>
       </c>
       <c r="L271" t="n">
-        <v>0.332</v>
+        <v>0.3403</v>
       </c>
       <c r="M271" t="n">
         <v>164</v>
@@ -15312,22 +15312,22 @@
         </is>
       </c>
       <c r="G276" t="n">
-        <v>0.3387</v>
+        <v>0.3343</v>
       </c>
       <c r="H276" t="n">
         <v>0.1821</v>
       </c>
       <c r="I276" t="n">
-        <v>0.2604</v>
+        <v>0.2582</v>
       </c>
       <c r="J276" t="n">
-        <v>0.6613</v>
+        <v>0.6657</v>
       </c>
       <c r="K276" t="n">
         <v>0.8179</v>
       </c>
       <c r="L276" t="n">
-        <v>0.7396</v>
+        <v>0.7418</v>
       </c>
       <c r="M276" t="n">
         <v>164</v>
@@ -15690,22 +15690,22 @@
         </is>
       </c>
       <c r="G283" t="n">
-        <v>0.4772</v>
+        <v>0.4614</v>
       </c>
       <c r="H283" t="n">
-        <v>0.319</v>
+        <v>0.2904</v>
       </c>
       <c r="I283" t="n">
-        <v>0.3981</v>
+        <v>0.3759</v>
       </c>
       <c r="J283" t="n">
-        <v>0.5228</v>
+        <v>0.5386</v>
       </c>
       <c r="K283" t="n">
-        <v>0.681</v>
+        <v>0.7096</v>
       </c>
       <c r="L283" t="n">
-        <v>0.6019</v>
+        <v>0.6241</v>
       </c>
       <c r="M283" t="n">
         <v>164</v>
@@ -15960,22 +15960,22 @@
         </is>
       </c>
       <c r="G288" t="n">
-        <v>0.5396</v>
+        <v>0.5349</v>
       </c>
       <c r="H288" t="n">
-        <v>0.3792</v>
+        <v>0.36</v>
       </c>
       <c r="I288" t="n">
-        <v>0.4594</v>
+        <v>0.4474</v>
       </c>
       <c r="J288" t="n">
-        <v>0.4604</v>
+        <v>0.4651</v>
       </c>
       <c r="K288" t="n">
-        <v>0.6208</v>
+        <v>0.64</v>
       </c>
       <c r="L288" t="n">
-        <v>0.5406</v>
+        <v>0.5526</v>
       </c>
       <c r="M288" t="n">
         <v>164</v>
@@ -16608,22 +16608,22 @@
         </is>
       </c>
       <c r="G300" t="n">
-        <v>0.2798</v>
+        <v>0.2742</v>
       </c>
       <c r="H300" t="n">
-        <v>0.1616</v>
+        <v>0.1583</v>
       </c>
       <c r="I300" t="n">
-        <v>0.2207</v>
+        <v>0.2162</v>
       </c>
       <c r="J300" t="n">
-        <v>0.7202</v>
+        <v>0.7258</v>
       </c>
       <c r="K300" t="n">
-        <v>0.8384</v>
+        <v>0.8417</v>
       </c>
       <c r="L300" t="n">
-        <v>0.7793</v>
+        <v>0.7838000000000001</v>
       </c>
       <c r="M300" t="n">
         <v>164</v>
@@ -16824,22 +16824,22 @@
         </is>
       </c>
       <c r="G304" t="n">
-        <v>0.8295</v>
+        <v>0.8196</v>
       </c>
       <c r="H304" t="n">
-        <v>0.7016</v>
+        <v>0.6956</v>
       </c>
       <c r="I304" t="n">
-        <v>0.7655</v>
+        <v>0.7576000000000001</v>
       </c>
       <c r="J304" t="n">
-        <v>0.1705</v>
+        <v>0.1804</v>
       </c>
       <c r="K304" t="n">
-        <v>0.2984</v>
+        <v>0.3044</v>
       </c>
       <c r="L304" t="n">
-        <v>0.2345</v>
+        <v>0.2424</v>
       </c>
       <c r="M304" t="n">
         <v>164</v>
@@ -17472,22 +17472,22 @@
         </is>
       </c>
       <c r="G316" t="n">
-        <v>0.6016</v>
+        <v>0.5985</v>
       </c>
       <c r="H316" t="n">
-        <v>0.44</v>
+        <v>0.4231</v>
       </c>
       <c r="I316" t="n">
-        <v>0.5208</v>
+        <v>0.5108</v>
       </c>
       <c r="J316" t="n">
-        <v>0.3984</v>
+        <v>0.4015</v>
       </c>
       <c r="K316" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5769</v>
       </c>
       <c r="L316" t="n">
-        <v>0.4792</v>
+        <v>0.4892</v>
       </c>
       <c r="M316" t="n">
         <v>164</v>
@@ -17634,22 +17634,22 @@
         </is>
       </c>
       <c r="G319" t="n">
-        <v>0.4699</v>
+        <v>0.4548</v>
       </c>
       <c r="H319" t="n">
-        <v>0.2896</v>
+        <v>0.2862</v>
       </c>
       <c r="I319" t="n">
-        <v>0.3798</v>
+        <v>0.3705</v>
       </c>
       <c r="J319" t="n">
-        <v>0.5301</v>
+        <v>0.5452</v>
       </c>
       <c r="K319" t="n">
-        <v>0.7104</v>
+        <v>0.7138</v>
       </c>
       <c r="L319" t="n">
-        <v>0.6202</v>
+        <v>0.6294999999999999</v>
       </c>
       <c r="M319" t="n">
         <v>164</v>
@@ -18282,22 +18282,22 @@
         </is>
       </c>
       <c r="G331" t="n">
-        <v>0.2213</v>
+        <v>0.2131</v>
       </c>
       <c r="H331" t="n">
-        <v>0.1319</v>
+        <v>0.1278</v>
       </c>
       <c r="I331" t="n">
-        <v>0.1766</v>
+        <v>0.1704</v>
       </c>
       <c r="J331" t="n">
-        <v>0.7786999999999999</v>
+        <v>0.7869</v>
       </c>
       <c r="K331" t="n">
-        <v>0.8681</v>
+        <v>0.8722</v>
       </c>
       <c r="L331" t="n">
-        <v>0.8234</v>
+        <v>0.8296</v>
       </c>
       <c r="M331" t="n">
         <v>164</v>
@@ -18390,22 +18390,22 @@
         </is>
       </c>
       <c r="G333" t="n">
-        <v>0.8334</v>
+        <v>0.8288</v>
       </c>
       <c r="H333" t="n">
-        <v>0.7353</v>
+        <v>0.7335</v>
       </c>
       <c r="I333" t="n">
-        <v>0.7844</v>
+        <v>0.7812</v>
       </c>
       <c r="J333" t="n">
-        <v>0.1666</v>
+        <v>0.1712</v>
       </c>
       <c r="K333" t="n">
-        <v>0.2647</v>
+        <v>0.2665</v>
       </c>
       <c r="L333" t="n">
-        <v>0.2156</v>
+        <v>0.2188</v>
       </c>
       <c r="M333" t="n">
         <v>164</v>
@@ -18501,19 +18501,19 @@
         <v>0.7374000000000001</v>
       </c>
       <c r="H335" t="n">
-        <v>0.5726</v>
+        <v>0.5707</v>
       </c>
       <c r="I335" t="n">
-        <v>0.655</v>
+        <v>0.654</v>
       </c>
       <c r="J335" t="n">
         <v>0.2626</v>
       </c>
       <c r="K335" t="n">
-        <v>0.4274</v>
+        <v>0.4293</v>
       </c>
       <c r="L335" t="n">
-        <v>0.345</v>
+        <v>0.346</v>
       </c>
       <c r="M335" t="n">
         <v>164</v>
@@ -18552,22 +18552,22 @@
         </is>
       </c>
       <c r="G336" t="n">
-        <v>0.7637</v>
+        <v>0.7667</v>
       </c>
       <c r="H336" t="n">
         <v>0.5982</v>
       </c>
       <c r="I336" t="n">
-        <v>0.6808999999999999</v>
+        <v>0.6824</v>
       </c>
       <c r="J336" t="n">
-        <v>0.2363</v>
+        <v>0.2333</v>
       </c>
       <c r="K336" t="n">
         <v>0.4018</v>
       </c>
       <c r="L336" t="n">
-        <v>0.3191</v>
+        <v>0.3176</v>
       </c>
       <c r="M336" t="n">
         <v>164</v>
@@ -18876,22 +18876,22 @@
         </is>
       </c>
       <c r="G342" t="n">
-        <v>0.8774999999999999</v>
+        <v>0.878</v>
       </c>
       <c r="H342" t="n">
         <v>0.7451</v>
       </c>
       <c r="I342" t="n">
-        <v>0.8113</v>
+        <v>0.8116</v>
       </c>
       <c r="J342" t="n">
-        <v>0.1225</v>
+        <v>0.122</v>
       </c>
       <c r="K342" t="n">
         <v>0.2549</v>
       </c>
       <c r="L342" t="n">
-        <v>0.1887</v>
+        <v>0.1884</v>
       </c>
       <c r="M342" t="n">
         <v>164</v>
@@ -19038,22 +19038,22 @@
         </is>
       </c>
       <c r="G345" t="n">
-        <v>0.6089</v>
+        <v>0.5909</v>
       </c>
       <c r="H345" t="n">
-        <v>0.4811</v>
+        <v>0.4692</v>
       </c>
       <c r="I345" t="n">
-        <v>0.545</v>
+        <v>0.53</v>
       </c>
       <c r="J345" t="n">
-        <v>0.3911</v>
+        <v>0.4091</v>
       </c>
       <c r="K345" t="n">
-        <v>0.5189</v>
+        <v>0.5308</v>
       </c>
       <c r="L345" t="n">
-        <v>0.455</v>
+        <v>0.47</v>
       </c>
       <c r="M345" t="n">
         <v>164</v>
@@ -19092,22 +19092,22 @@
         </is>
       </c>
       <c r="G346" t="n">
-        <v>0.7249</v>
+        <v>0.7181999999999999</v>
       </c>
       <c r="H346" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.5491</v>
       </c>
       <c r="I346" t="n">
-        <v>0.6449</v>
+        <v>0.6337</v>
       </c>
       <c r="J346" t="n">
-        <v>0.2751</v>
+        <v>0.2818</v>
       </c>
       <c r="K346" t="n">
-        <v>0.435</v>
+        <v>0.4509</v>
       </c>
       <c r="L346" t="n">
-        <v>0.3551</v>
+        <v>0.3663</v>
       </c>
       <c r="M346" t="n">
         <v>164</v>
@@ -19308,22 +19308,22 @@
         </is>
       </c>
       <c r="G350" t="n">
-        <v>0.785</v>
+        <v>0.7889</v>
       </c>
       <c r="H350" t="n">
         <v>0.6461</v>
       </c>
       <c r="I350" t="n">
-        <v>0.7156</v>
+        <v>0.7175</v>
       </c>
       <c r="J350" t="n">
-        <v>0.215</v>
+        <v>0.2111</v>
       </c>
       <c r="K350" t="n">
         <v>0.3539</v>
       </c>
       <c r="L350" t="n">
-        <v>0.2844</v>
+        <v>0.2825</v>
       </c>
       <c r="M350" t="n">
         <v>164</v>
@@ -19740,22 +19740,22 @@
         </is>
       </c>
       <c r="G358" t="n">
-        <v>0.419</v>
+        <v>0.4155</v>
       </c>
       <c r="H358" t="n">
-        <v>0.2654</v>
+        <v>0.2487</v>
       </c>
       <c r="I358" t="n">
-        <v>0.3422</v>
+        <v>0.3321</v>
       </c>
       <c r="J358" t="n">
-        <v>0.581</v>
+        <v>0.5845</v>
       </c>
       <c r="K358" t="n">
-        <v>0.7346</v>
+        <v>0.7513</v>
       </c>
       <c r="L358" t="n">
-        <v>0.6578000000000001</v>
+        <v>0.6679</v>
       </c>
       <c r="M358" t="n">
         <v>164</v>
@@ -19794,22 +19794,22 @@
         </is>
       </c>
       <c r="G359" t="n">
-        <v>0.3723</v>
+        <v>0.3785</v>
       </c>
       <c r="H359" t="n">
-        <v>0.2228</v>
+        <v>0.2258</v>
       </c>
       <c r="I359" t="n">
-        <v>0.2976</v>
+        <v>0.3022</v>
       </c>
       <c r="J359" t="n">
-        <v>0.6277</v>
+        <v>0.6215000000000001</v>
       </c>
       <c r="K359" t="n">
-        <v>0.7772</v>
+        <v>0.7742</v>
       </c>
       <c r="L359" t="n">
-        <v>0.7024</v>
+        <v>0.6978</v>
       </c>
       <c r="M359" t="n">
         <v>164</v>
@@ -19848,22 +19848,22 @@
         </is>
       </c>
       <c r="G360" t="n">
-        <v>0.3694</v>
+        <v>0.3739</v>
       </c>
       <c r="H360" t="n">
-        <v>0.2274</v>
+        <v>0.2491</v>
       </c>
       <c r="I360" t="n">
-        <v>0.2984</v>
+        <v>0.3115</v>
       </c>
       <c r="J360" t="n">
-        <v>0.6306</v>
+        <v>0.6261</v>
       </c>
       <c r="K360" t="n">
-        <v>0.7726</v>
+        <v>0.7509</v>
       </c>
       <c r="L360" t="n">
-        <v>0.7016</v>
+        <v>0.6885</v>
       </c>
       <c r="M360" t="n">
         <v>164</v>
@@ -19902,22 +19902,22 @@
         </is>
       </c>
       <c r="G361" t="n">
-        <v>0.42</v>
+        <v>0.4182</v>
       </c>
       <c r="H361" t="n">
-        <v>0.2698</v>
+        <v>0.2808</v>
       </c>
       <c r="I361" t="n">
-        <v>0.3449</v>
+        <v>0.3495</v>
       </c>
       <c r="J361" t="n">
-        <v>0.58</v>
+        <v>0.5818</v>
       </c>
       <c r="K361" t="n">
-        <v>0.7302</v>
+        <v>0.7192</v>
       </c>
       <c r="L361" t="n">
-        <v>0.6551</v>
+        <v>0.6505</v>
       </c>
       <c r="M361" t="n">
         <v>164</v>
@@ -19956,22 +19956,22 @@
         </is>
       </c>
       <c r="G362" t="n">
-        <v>0.6756</v>
+        <v>0.6793</v>
       </c>
       <c r="H362" t="n">
-        <v>0.5605</v>
+        <v>0.5701000000000001</v>
       </c>
       <c r="I362" t="n">
-        <v>0.618</v>
+        <v>0.6247</v>
       </c>
       <c r="J362" t="n">
-        <v>0.3244</v>
+        <v>0.3207</v>
       </c>
       <c r="K362" t="n">
-        <v>0.4395</v>
+        <v>0.4299</v>
       </c>
       <c r="L362" t="n">
-        <v>0.382</v>
+        <v>0.3753</v>
       </c>
       <c r="M362" t="n">
         <v>164</v>
@@ -20010,22 +20010,22 @@
         </is>
       </c>
       <c r="G363" t="n">
-        <v>0.2528</v>
+        <v>0.2611</v>
       </c>
       <c r="H363" t="n">
-        <v>0.1386</v>
+        <v>0.1414</v>
       </c>
       <c r="I363" t="n">
-        <v>0.1957</v>
+        <v>0.2012</v>
       </c>
       <c r="J363" t="n">
-        <v>0.7472</v>
+        <v>0.7389</v>
       </c>
       <c r="K363" t="n">
-        <v>0.8614000000000001</v>
+        <v>0.8586</v>
       </c>
       <c r="L363" t="n">
-        <v>0.8043</v>
+        <v>0.7988</v>
       </c>
       <c r="M363" t="n">
         <v>164</v>
@@ -20064,22 +20064,22 @@
         </is>
       </c>
       <c r="G364" t="n">
-        <v>0.2504</v>
+        <v>0.2557</v>
       </c>
       <c r="H364" t="n">
-        <v>0.1335</v>
+        <v>0.134</v>
       </c>
       <c r="I364" t="n">
-        <v>0.192</v>
+        <v>0.1948</v>
       </c>
       <c r="J364" t="n">
-        <v>0.7496</v>
+        <v>0.7443</v>
       </c>
       <c r="K364" t="n">
-        <v>0.8665</v>
+        <v>0.866</v>
       </c>
       <c r="L364" t="n">
-        <v>0.8080000000000001</v>
+        <v>0.8052</v>
       </c>
       <c r="M364" t="n">
         <v>164</v>
@@ -20118,22 +20118,22 @@
         </is>
       </c>
       <c r="G365" t="n">
-        <v>0.3394</v>
+        <v>0.3506</v>
       </c>
       <c r="H365" t="n">
-        <v>0.2203</v>
+        <v>0.2243</v>
       </c>
       <c r="I365" t="n">
-        <v>0.2798</v>
+        <v>0.2874</v>
       </c>
       <c r="J365" t="n">
-        <v>0.6606</v>
+        <v>0.6494</v>
       </c>
       <c r="K365" t="n">
-        <v>0.7796999999999999</v>
+        <v>0.7756999999999999</v>
       </c>
       <c r="L365" t="n">
-        <v>0.7202</v>
+        <v>0.7126</v>
       </c>
       <c r="M365" t="n">
         <v>164</v>
@@ -20172,22 +20172,22 @@
         </is>
       </c>
       <c r="G366" t="n">
-        <v>0.6364</v>
+        <v>0.6505</v>
       </c>
       <c r="H366" t="n">
-        <v>0.5403</v>
+        <v>0.5423</v>
       </c>
       <c r="I366" t="n">
-        <v>0.5883</v>
+        <v>0.5964</v>
       </c>
       <c r="J366" t="n">
-        <v>0.3636</v>
+        <v>0.3495</v>
       </c>
       <c r="K366" t="n">
-        <v>0.4597</v>
+        <v>0.4577</v>
       </c>
       <c r="L366" t="n">
-        <v>0.4117</v>
+        <v>0.4036</v>
       </c>
       <c r="M366" t="n">
         <v>164</v>
@@ -20226,22 +20226,22 @@
         </is>
       </c>
       <c r="G367" t="n">
-        <v>0.618</v>
+        <v>0.622</v>
       </c>
       <c r="H367" t="n">
-        <v>0.4833</v>
+        <v>0.4968</v>
       </c>
       <c r="I367" t="n">
-        <v>0.5506</v>
+        <v>0.5594</v>
       </c>
       <c r="J367" t="n">
-        <v>0.382</v>
+        <v>0.378</v>
       </c>
       <c r="K367" t="n">
-        <v>0.5167</v>
+        <v>0.5032</v>
       </c>
       <c r="L367" t="n">
-        <v>0.4494</v>
+        <v>0.4406</v>
       </c>
       <c r="M367" t="n">
         <v>164</v>
@@ -20280,22 +20280,22 @@
         </is>
       </c>
       <c r="G368" t="n">
-        <v>0.7256</v>
+        <v>0.7331</v>
       </c>
       <c r="H368" t="n">
-        <v>0.59</v>
+        <v>0.5996</v>
       </c>
       <c r="I368" t="n">
-        <v>0.6578000000000001</v>
+        <v>0.6664</v>
       </c>
       <c r="J368" t="n">
-        <v>0.2744</v>
+        <v>0.2669</v>
       </c>
       <c r="K368" t="n">
-        <v>0.41</v>
+        <v>0.4004</v>
       </c>
       <c r="L368" t="n">
-        <v>0.3422</v>
+        <v>0.3336</v>
       </c>
       <c r="M368" t="n">
         <v>164</v>
@@ -20334,22 +20334,22 @@
         </is>
       </c>
       <c r="G369" t="n">
-        <v>0.3017</v>
+        <v>0.3175</v>
       </c>
       <c r="H369" t="n">
-        <v>0.2099</v>
+        <v>0.2194</v>
       </c>
       <c r="I369" t="n">
-        <v>0.2558</v>
+        <v>0.2684</v>
       </c>
       <c r="J369" t="n">
-        <v>0.6983</v>
+        <v>0.6825</v>
       </c>
       <c r="K369" t="n">
-        <v>0.7901</v>
+        <v>0.7806</v>
       </c>
       <c r="L369" t="n">
-        <v>0.7442</v>
+        <v>0.7316</v>
       </c>
       <c r="M369" t="n">
         <v>164</v>
@@ -20391,19 +20391,19 @@
         <v>0.2964</v>
       </c>
       <c r="H370" t="n">
-        <v>0.1775</v>
+        <v>0.175</v>
       </c>
       <c r="I370" t="n">
-        <v>0.237</v>
+        <v>0.2357</v>
       </c>
       <c r="J370" t="n">
         <v>0.7036</v>
       </c>
       <c r="K370" t="n">
-        <v>0.8225</v>
+        <v>0.825</v>
       </c>
       <c r="L370" t="n">
-        <v>0.763</v>
+        <v>0.7643</v>
       </c>
       <c r="M370" t="n">
         <v>164</v>
@@ -20874,22 +20874,22 @@
         </is>
       </c>
       <c r="G379" t="n">
-        <v>0.8475</v>
+        <v>0.8514</v>
       </c>
       <c r="H379" t="n">
         <v>0.7551</v>
       </c>
       <c r="I379" t="n">
-        <v>0.8013</v>
+        <v>0.8032</v>
       </c>
       <c r="J379" t="n">
-        <v>0.1525</v>
+        <v>0.1486</v>
       </c>
       <c r="K379" t="n">
         <v>0.2449</v>
       </c>
       <c r="L379" t="n">
-        <v>0.1987</v>
+        <v>0.1968</v>
       </c>
       <c r="M379" t="n">
         <v>164</v>
@@ -20982,22 +20982,22 @@
         </is>
       </c>
       <c r="G381" t="n">
-        <v>0.5135</v>
+        <v>0.4838</v>
       </c>
       <c r="H381" t="n">
-        <v>0.3318</v>
+        <v>0.3316</v>
       </c>
       <c r="I381" t="n">
-        <v>0.4226</v>
+        <v>0.4077</v>
       </c>
       <c r="J381" t="n">
-        <v>0.4865</v>
+        <v>0.5162</v>
       </c>
       <c r="K381" t="n">
-        <v>0.6682</v>
+        <v>0.6684</v>
       </c>
       <c r="L381" t="n">
-        <v>0.5774</v>
+        <v>0.5923</v>
       </c>
       <c r="M381" t="n">
         <v>164</v>
@@ -21522,22 +21522,22 @@
         </is>
       </c>
       <c r="G391" t="n">
-        <v>0.471</v>
+        <v>0.4594</v>
       </c>
       <c r="H391" t="n">
-        <v>0.3493</v>
+        <v>0.3171</v>
       </c>
       <c r="I391" t="n">
-        <v>0.4102</v>
+        <v>0.3882</v>
       </c>
       <c r="J391" t="n">
-        <v>0.529</v>
+        <v>0.5406</v>
       </c>
       <c r="K391" t="n">
-        <v>0.6506999999999999</v>
+        <v>0.6829</v>
       </c>
       <c r="L391" t="n">
-        <v>0.5898</v>
+        <v>0.6118</v>
       </c>
       <c r="M391" t="n">
         <v>164</v>
@@ -22008,22 +22008,22 @@
         </is>
       </c>
       <c r="G400" t="n">
-        <v>0.4405</v>
+        <v>0.4347</v>
       </c>
       <c r="H400" t="n">
-        <v>0.2798</v>
+        <v>0.2752</v>
       </c>
       <c r="I400" t="n">
-        <v>0.3601</v>
+        <v>0.355</v>
       </c>
       <c r="J400" t="n">
-        <v>0.5595</v>
+        <v>0.5653</v>
       </c>
       <c r="K400" t="n">
-        <v>0.7202</v>
+        <v>0.7248</v>
       </c>
       <c r="L400" t="n">
-        <v>0.6399</v>
+        <v>0.645</v>
       </c>
       <c r="M400" t="n">
         <v>164</v>
@@ -22440,22 +22440,22 @@
         </is>
       </c>
       <c r="G408" t="n">
-        <v>0.2348</v>
+        <v>0.2298</v>
       </c>
       <c r="H408" t="n">
-        <v>0.1346</v>
+        <v>0.1318</v>
       </c>
       <c r="I408" t="n">
-        <v>0.1847</v>
+        <v>0.1808</v>
       </c>
       <c r="J408" t="n">
-        <v>0.7652</v>
+        <v>0.7702</v>
       </c>
       <c r="K408" t="n">
-        <v>0.8653999999999999</v>
+        <v>0.8682</v>
       </c>
       <c r="L408" t="n">
-        <v>0.8153</v>
+        <v>0.8192</v>
       </c>
       <c r="M408" t="n">
         <v>164</v>
@@ -22818,22 +22818,22 @@
         </is>
       </c>
       <c r="G415" t="n">
-        <v>0.7343</v>
+        <v>0.7226</v>
       </c>
       <c r="H415" t="n">
-        <v>0.5957</v>
+        <v>0.5824</v>
       </c>
       <c r="I415" t="n">
-        <v>0.665</v>
+        <v>0.6525</v>
       </c>
       <c r="J415" t="n">
-        <v>0.2657</v>
+        <v>0.2774</v>
       </c>
       <c r="K415" t="n">
-        <v>0.4043</v>
+        <v>0.4176</v>
       </c>
       <c r="L415" t="n">
-        <v>0.335</v>
+        <v>0.3475</v>
       </c>
       <c r="M415" t="n">
         <v>164</v>
@@ -23142,22 +23142,22 @@
         </is>
       </c>
       <c r="G421" t="n">
-        <v>0.7534</v>
+        <v>0.7459</v>
       </c>
       <c r="H421" t="n">
-        <v>0.6343</v>
+        <v>0.6191</v>
       </c>
       <c r="I421" t="n">
-        <v>0.6938</v>
+        <v>0.6825</v>
       </c>
       <c r="J421" t="n">
-        <v>0.2466</v>
+        <v>0.2541</v>
       </c>
       <c r="K421" t="n">
-        <v>0.3657</v>
+        <v>0.3809</v>
       </c>
       <c r="L421" t="n">
-        <v>0.3062</v>
+        <v>0.3175</v>
       </c>
       <c r="M421" t="n">
         <v>164</v>
@@ -23412,22 +23412,22 @@
         </is>
       </c>
       <c r="G426" t="n">
-        <v>0.4991</v>
+        <v>0.4814</v>
       </c>
       <c r="H426" t="n">
-        <v>0.3611</v>
+        <v>0.3489</v>
       </c>
       <c r="I426" t="n">
-        <v>0.4301</v>
+        <v>0.4152</v>
       </c>
       <c r="J426" t="n">
-        <v>0.5009</v>
+        <v>0.5185999999999999</v>
       </c>
       <c r="K426" t="n">
-        <v>0.6389</v>
+        <v>0.6511</v>
       </c>
       <c r="L426" t="n">
-        <v>0.5699</v>
+        <v>0.5848</v>
       </c>
       <c r="M426" t="n">
         <v>164</v>
@@ -23628,22 +23628,22 @@
         </is>
       </c>
       <c r="G430" t="n">
-        <v>0.2713</v>
+        <v>0.2613</v>
       </c>
       <c r="H430" t="n">
-        <v>0.139</v>
+        <v>0.1323</v>
       </c>
       <c r="I430" t="n">
-        <v>0.2052</v>
+        <v>0.1968</v>
       </c>
       <c r="J430" t="n">
-        <v>0.7287</v>
+        <v>0.7387</v>
       </c>
       <c r="K430" t="n">
-        <v>0.861</v>
+        <v>0.8677</v>
       </c>
       <c r="L430" t="n">
-        <v>0.7948</v>
+        <v>0.8032</v>
       </c>
       <c r="M430" t="n">
         <v>164</v>
@@ -23736,22 +23736,22 @@
         </is>
       </c>
       <c r="G432" t="n">
-        <v>0.2767</v>
+        <v>0.2733</v>
       </c>
       <c r="H432" t="n">
         <v>0.1576</v>
       </c>
       <c r="I432" t="n">
-        <v>0.2172</v>
+        <v>0.2154</v>
       </c>
       <c r="J432" t="n">
-        <v>0.7233000000000001</v>
+        <v>0.7267</v>
       </c>
       <c r="K432" t="n">
         <v>0.8424</v>
       </c>
       <c r="L432" t="n">
-        <v>0.7828000000000001</v>
+        <v>0.7846</v>
       </c>
       <c r="M432" t="n">
         <v>164</v>
@@ -23790,22 +23790,22 @@
         </is>
       </c>
       <c r="G433" t="n">
-        <v>0.284</v>
+        <v>0.2741</v>
       </c>
       <c r="H433" t="n">
-        <v>0.1524</v>
+        <v>0.1409</v>
       </c>
       <c r="I433" t="n">
-        <v>0.2182</v>
+        <v>0.2075</v>
       </c>
       <c r="J433" t="n">
-        <v>0.716</v>
+        <v>0.7259</v>
       </c>
       <c r="K433" t="n">
-        <v>0.8476</v>
+        <v>0.8591</v>
       </c>
       <c r="L433" t="n">
-        <v>0.7818000000000001</v>
+        <v>0.7925</v>
       </c>
       <c r="M433" t="n">
         <v>164</v>
@@ -23898,22 +23898,22 @@
         </is>
       </c>
       <c r="G435" t="n">
-        <v>0.2283</v>
+        <v>0.2191</v>
       </c>
       <c r="H435" t="n">
-        <v>0.1307</v>
+        <v>0.1302</v>
       </c>
       <c r="I435" t="n">
-        <v>0.1795</v>
+        <v>0.1746</v>
       </c>
       <c r="J435" t="n">
-        <v>0.7717000000000001</v>
+        <v>0.7809</v>
       </c>
       <c r="K435" t="n">
-        <v>0.8693</v>
+        <v>0.8698</v>
       </c>
       <c r="L435" t="n">
-        <v>0.8205</v>
+        <v>0.8254</v>
       </c>
       <c r="M435" t="n">
         <v>164</v>
@@ -23952,22 +23952,22 @@
         </is>
       </c>
       <c r="G436" t="n">
-        <v>0.5849</v>
+        <v>0.5799</v>
       </c>
       <c r="H436" t="n">
-        <v>0.4543</v>
+        <v>0.4298</v>
       </c>
       <c r="I436" t="n">
-        <v>0.5196</v>
+        <v>0.5048</v>
       </c>
       <c r="J436" t="n">
-        <v>0.4151</v>
+        <v>0.4201</v>
       </c>
       <c r="K436" t="n">
-        <v>0.5457</v>
+        <v>0.5702</v>
       </c>
       <c r="L436" t="n">
-        <v>0.4804</v>
+        <v>0.4952</v>
       </c>
       <c r="M436" t="n">
         <v>164</v>

</xml_diff>

<commit_message>
Update NBA sim outputs (2026-04-18)
</commit_message>
<xml_diff>
--- a/nba/public/data/nba_matchup_probs.xlsx
+++ b/nba/public/data/nba_matchup_probs.xlsx
@@ -839,22 +839,22 @@
         <v>48</v>
       </c>
       <c r="G6">
-        <v>0.8365</v>
+        <v>0.8413</v>
       </c>
       <c r="H6">
         <v>0.7193000000000001</v>
       </c>
       <c r="I6">
-        <v>0.7779</v>
+        <v>0.7803</v>
       </c>
       <c r="J6">
-        <v>0.1635</v>
+        <v>0.1587</v>
       </c>
       <c r="K6">
         <v>0.2807</v>
       </c>
       <c r="L6">
-        <v>0.2221</v>
+        <v>0.2197</v>
       </c>
       <c r="M6">
         <v>179</v>
@@ -1015,22 +1015,22 @@
         <v>52</v>
       </c>
       <c r="G10">
-        <v>0.6209</v>
+        <v>0.628</v>
       </c>
       <c r="H10">
-        <v>0.4756</v>
+        <v>0.4776</v>
       </c>
       <c r="I10">
-        <v>0.5482</v>
+        <v>0.5528</v>
       </c>
       <c r="J10">
-        <v>0.3791</v>
+        <v>0.372</v>
       </c>
       <c r="K10">
-        <v>0.5244</v>
+        <v>0.5224</v>
       </c>
       <c r="L10">
-        <v>0.4518</v>
+        <v>0.4472</v>
       </c>
       <c r="M10">
         <v>179</v>
@@ -1323,22 +1323,22 @@
         <v>59</v>
       </c>
       <c r="G17">
-        <v>0.6828</v>
+        <v>0.6865</v>
       </c>
       <c r="H17">
-        <v>0.5212</v>
+        <v>0.5259</v>
       </c>
       <c r="I17">
-        <v>0.602</v>
+        <v>0.6062</v>
       </c>
       <c r="J17">
-        <v>0.3172</v>
+        <v>0.3135</v>
       </c>
       <c r="K17">
-        <v>0.4788</v>
+        <v>0.4741</v>
       </c>
       <c r="L17">
-        <v>0.398</v>
+        <v>0.3938</v>
       </c>
       <c r="M17">
         <v>179</v>
@@ -1367,22 +1367,22 @@
         <v>60</v>
       </c>
       <c r="G18">
-        <v>0.8187</v>
+        <v>0.8217</v>
       </c>
       <c r="H18">
         <v>0.7007</v>
       </c>
       <c r="I18">
-        <v>0.7597</v>
+        <v>0.7612</v>
       </c>
       <c r="J18">
-        <v>0.1813</v>
+        <v>0.1783</v>
       </c>
       <c r="K18">
         <v>0.2993</v>
       </c>
       <c r="L18">
-        <v>0.2403</v>
+        <v>0.2388</v>
       </c>
       <c r="M18">
         <v>179</v>
@@ -1455,22 +1455,22 @@
         <v>62</v>
       </c>
       <c r="G20">
-        <v>0.6455</v>
+        <v>0.6545</v>
       </c>
       <c r="H20">
         <v>0.485</v>
       </c>
       <c r="I20">
-        <v>0.5652</v>
+        <v>0.5698</v>
       </c>
       <c r="J20">
-        <v>0.3545</v>
+        <v>0.3455</v>
       </c>
       <c r="K20">
         <v>0.515</v>
       </c>
       <c r="L20">
-        <v>0.4348</v>
+        <v>0.4302</v>
       </c>
       <c r="M20">
         <v>179</v>
@@ -1499,22 +1499,22 @@
         <v>63</v>
       </c>
       <c r="G21">
-        <v>0.6454</v>
+        <v>0.6761</v>
       </c>
       <c r="H21">
-        <v>0.508</v>
+        <v>0.5172</v>
       </c>
       <c r="I21">
-        <v>0.5767</v>
+        <v>0.5966</v>
       </c>
       <c r="J21">
-        <v>0.3546</v>
+        <v>0.3239</v>
       </c>
       <c r="K21">
-        <v>0.492</v>
+        <v>0.4828</v>
       </c>
       <c r="L21">
-        <v>0.4233</v>
+        <v>0.4034</v>
       </c>
       <c r="M21">
         <v>179</v>
@@ -1675,22 +1675,22 @@
         <v>67</v>
       </c>
       <c r="G25">
-        <v>0.5867</v>
+        <v>0.6022999999999999</v>
       </c>
       <c r="H25">
-        <v>0.4636</v>
+        <v>0.4654</v>
       </c>
       <c r="I25">
-        <v>0.5252</v>
+        <v>0.5338000000000001</v>
       </c>
       <c r="J25">
-        <v>0.4133</v>
+        <v>0.3977</v>
       </c>
       <c r="K25">
-        <v>0.5364</v>
+        <v>0.5346</v>
       </c>
       <c r="L25">
-        <v>0.4748</v>
+        <v>0.4662</v>
       </c>
       <c r="M25">
         <v>179</v>
@@ -1895,7 +1895,7 @@
         <v>73</v>
       </c>
       <c r="G30">
-        <v>0.5824</v>
+        <v>0.5822000000000001</v>
       </c>
       <c r="H30">
         <v>0.4397</v>
@@ -1904,7 +1904,7 @@
         <v>0.511</v>
       </c>
       <c r="J30">
-        <v>0.4176</v>
+        <v>0.4178</v>
       </c>
       <c r="K30">
         <v>0.5603</v>
@@ -2027,22 +2027,22 @@
         <v>47</v>
       </c>
       <c r="G33">
-        <v>0.8819</v>
+        <v>0.884</v>
       </c>
       <c r="H33">
         <v>0.759</v>
       </c>
       <c r="I33">
-        <v>0.8204</v>
+        <v>0.8215</v>
       </c>
       <c r="J33">
-        <v>0.1181</v>
+        <v>0.116</v>
       </c>
       <c r="K33">
         <v>0.241</v>
       </c>
       <c r="L33">
-        <v>0.1796</v>
+        <v>0.1785</v>
       </c>
       <c r="M33">
         <v>179</v>
@@ -2247,22 +2247,22 @@
         <v>52</v>
       </c>
       <c r="G38">
-        <v>0.746</v>
+        <v>0.7502</v>
       </c>
       <c r="H38">
         <v>0.5906</v>
       </c>
       <c r="I38">
-        <v>0.6683</v>
+        <v>0.6704</v>
       </c>
       <c r="J38">
-        <v>0.254</v>
+        <v>0.2498</v>
       </c>
       <c r="K38">
         <v>0.4094</v>
       </c>
       <c r="L38">
-        <v>0.3317</v>
+        <v>0.3296</v>
       </c>
       <c r="M38">
         <v>179</v>
@@ -2294,7 +2294,7 @@
         <v>0.7524</v>
       </c>
       <c r="H39">
-        <v>0.6121</v>
+        <v>0.6119</v>
       </c>
       <c r="I39">
         <v>0.6822</v>
@@ -2303,7 +2303,7 @@
         <v>0.2476</v>
       </c>
       <c r="K39">
-        <v>0.3879</v>
+        <v>0.3881</v>
       </c>
       <c r="L39">
         <v>0.3178</v>
@@ -2423,22 +2423,22 @@
         <v>56</v>
       </c>
       <c r="G42">
-        <v>0.7469</v>
+        <v>0.7501</v>
       </c>
       <c r="H42">
         <v>0.541</v>
       </c>
       <c r="I42">
-        <v>0.644</v>
+        <v>0.6456</v>
       </c>
       <c r="J42">
-        <v>0.2531</v>
+        <v>0.2499</v>
       </c>
       <c r="K42">
         <v>0.459</v>
       </c>
       <c r="L42">
-        <v>0.356</v>
+        <v>0.3544</v>
       </c>
       <c r="M42">
         <v>179</v>
@@ -2555,22 +2555,22 @@
         <v>59</v>
       </c>
       <c r="G45">
-        <v>0.7904</v>
+        <v>0.7969000000000001</v>
       </c>
       <c r="H45">
-        <v>0.6452</v>
+        <v>0.6489</v>
       </c>
       <c r="I45">
-        <v>0.7178</v>
+        <v>0.7229</v>
       </c>
       <c r="J45">
-        <v>0.2096</v>
+        <v>0.2031</v>
       </c>
       <c r="K45">
-        <v>0.3548</v>
+        <v>0.3511</v>
       </c>
       <c r="L45">
-        <v>0.2822</v>
+        <v>0.2771</v>
       </c>
       <c r="M45">
         <v>179</v>
@@ -2602,19 +2602,19 @@
         <v>0.87</v>
       </c>
       <c r="H46">
-        <v>0.7591</v>
+        <v>0.7635999999999999</v>
       </c>
       <c r="I46">
-        <v>0.8146</v>
+        <v>0.8168</v>
       </c>
       <c r="J46">
         <v>0.13</v>
       </c>
       <c r="K46">
-        <v>0.2409</v>
+        <v>0.2364</v>
       </c>
       <c r="L46">
-        <v>0.1854</v>
+        <v>0.1832</v>
       </c>
       <c r="M46">
         <v>179</v>
@@ -2646,19 +2646,19 @@
         <v>0.7841</v>
       </c>
       <c r="H47">
-        <v>0.6447000000000001</v>
+        <v>0.6403</v>
       </c>
       <c r="I47">
-        <v>0.7144</v>
+        <v>0.7122000000000001</v>
       </c>
       <c r="J47">
         <v>0.2159</v>
       </c>
       <c r="K47">
-        <v>0.3553</v>
+        <v>0.3597</v>
       </c>
       <c r="L47">
-        <v>0.2856</v>
+        <v>0.2878</v>
       </c>
       <c r="M47">
         <v>179</v>
@@ -2690,19 +2690,19 @@
         <v>0.7852</v>
       </c>
       <c r="H48">
-        <v>0.6405999999999999</v>
+        <v>0.6451</v>
       </c>
       <c r="I48">
-        <v>0.7129</v>
+        <v>0.7151</v>
       </c>
       <c r="J48">
         <v>0.2148</v>
       </c>
       <c r="K48">
-        <v>0.3594</v>
+        <v>0.3549</v>
       </c>
       <c r="L48">
-        <v>0.2871</v>
+        <v>0.2849</v>
       </c>
       <c r="M48">
         <v>179</v>
@@ -2731,22 +2731,22 @@
         <v>63</v>
       </c>
       <c r="G49">
-        <v>0.7717000000000001</v>
+        <v>0.7883</v>
       </c>
       <c r="H49">
-        <v>0.6344</v>
+        <v>0.6533</v>
       </c>
       <c r="I49">
-        <v>0.703</v>
+        <v>0.7208</v>
       </c>
       <c r="J49">
-        <v>0.2283</v>
+        <v>0.2117</v>
       </c>
       <c r="K49">
-        <v>0.3656</v>
+        <v>0.3467</v>
       </c>
       <c r="L49">
-        <v>0.297</v>
+        <v>0.2792</v>
       </c>
       <c r="M49">
         <v>179</v>
@@ -2866,19 +2866,19 @@
         <v>0.6432</v>
       </c>
       <c r="H52">
-        <v>0.4896</v>
+        <v>0.494</v>
       </c>
       <c r="I52">
-        <v>0.5664</v>
+        <v>0.5686</v>
       </c>
       <c r="J52">
         <v>0.3568</v>
       </c>
       <c r="K52">
-        <v>0.5104</v>
+        <v>0.506</v>
       </c>
       <c r="L52">
-        <v>0.4336</v>
+        <v>0.4314</v>
       </c>
       <c r="M52">
         <v>179</v>
@@ -2907,22 +2907,22 @@
         <v>67</v>
       </c>
       <c r="G53">
-        <v>0.7306</v>
+        <v>0.7444</v>
       </c>
       <c r="H53">
-        <v>0.5770999999999999</v>
+        <v>0.5805</v>
       </c>
       <c r="I53">
-        <v>0.6538</v>
+        <v>0.6624</v>
       </c>
       <c r="J53">
-        <v>0.2694</v>
+        <v>0.2556</v>
       </c>
       <c r="K53">
-        <v>0.4229</v>
+        <v>0.4195</v>
       </c>
       <c r="L53">
-        <v>0.3462</v>
+        <v>0.3376</v>
       </c>
       <c r="M53">
         <v>179</v>
@@ -3391,22 +3391,22 @@
         <v>51</v>
       </c>
       <c r="G64">
-        <v>0.6878</v>
+        <v>0.6891</v>
       </c>
       <c r="H64">
         <v>0.4954</v>
       </c>
       <c r="I64">
-        <v>0.5916</v>
+        <v>0.5923</v>
       </c>
       <c r="J64">
-        <v>0.3122</v>
+        <v>0.3109</v>
       </c>
       <c r="K64">
         <v>0.5046</v>
       </c>
       <c r="L64">
-        <v>0.4084</v>
+        <v>0.4077</v>
       </c>
       <c r="M64">
         <v>179</v>
@@ -3438,19 +3438,19 @@
         <v>0.7081</v>
       </c>
       <c r="H65">
-        <v>0.5655</v>
+        <v>0.5633</v>
       </c>
       <c r="I65">
-        <v>0.6368</v>
+        <v>0.6357</v>
       </c>
       <c r="J65">
         <v>0.2919</v>
       </c>
       <c r="K65">
-        <v>0.4345</v>
+        <v>0.4367</v>
       </c>
       <c r="L65">
-        <v>0.3632</v>
+        <v>0.3643</v>
       </c>
       <c r="M65">
         <v>179</v>
@@ -3523,22 +3523,22 @@
         <v>54</v>
       </c>
       <c r="G67">
-        <v>0.7764</v>
+        <v>0.7776999999999999</v>
       </c>
       <c r="H67">
         <v>0.5899</v>
       </c>
       <c r="I67">
-        <v>0.6831</v>
+        <v>0.6838</v>
       </c>
       <c r="J67">
-        <v>0.2236</v>
+        <v>0.2223</v>
       </c>
       <c r="K67">
         <v>0.4101</v>
       </c>
       <c r="L67">
-        <v>0.3169</v>
+        <v>0.3162</v>
       </c>
       <c r="M67">
         <v>179</v>
@@ -3614,19 +3614,19 @@
         <v>0.7064</v>
       </c>
       <c r="H69">
-        <v>0.5575</v>
+        <v>0.5628</v>
       </c>
       <c r="I69">
-        <v>0.632</v>
+        <v>0.6346000000000001</v>
       </c>
       <c r="J69">
         <v>0.2936</v>
       </c>
       <c r="K69">
-        <v>0.4425</v>
+        <v>0.4372</v>
       </c>
       <c r="L69">
-        <v>0.368</v>
+        <v>0.3654</v>
       </c>
       <c r="M69">
         <v>179</v>
@@ -3743,22 +3743,22 @@
         <v>59</v>
       </c>
       <c r="G72">
-        <v>0.7781</v>
+        <v>0.7794</v>
       </c>
       <c r="H72">
-        <v>0.5958</v>
+        <v>0.5981</v>
       </c>
       <c r="I72">
-        <v>0.6869</v>
+        <v>0.6888</v>
       </c>
       <c r="J72">
-        <v>0.2219</v>
+        <v>0.2206</v>
       </c>
       <c r="K72">
-        <v>0.4042</v>
+        <v>0.4019</v>
       </c>
       <c r="L72">
-        <v>0.3131</v>
+        <v>0.3112</v>
       </c>
       <c r="M72">
         <v>179</v>
@@ -3875,22 +3875,22 @@
         <v>62</v>
       </c>
       <c r="G75">
-        <v>0.762</v>
+        <v>0.7634</v>
       </c>
       <c r="H75">
         <v>0.5554</v>
       </c>
       <c r="I75">
-        <v>0.6587</v>
+        <v>0.6594</v>
       </c>
       <c r="J75">
-        <v>0.238</v>
+        <v>0.2366</v>
       </c>
       <c r="K75">
         <v>0.4446</v>
       </c>
       <c r="L75">
-        <v>0.3413</v>
+        <v>0.3406</v>
       </c>
       <c r="M75">
         <v>179</v>
@@ -3919,22 +3919,22 @@
         <v>63</v>
       </c>
       <c r="G76">
-        <v>0.7687</v>
+        <v>0.7852</v>
       </c>
       <c r="H76">
-        <v>0.599</v>
+        <v>0.6124000000000001</v>
       </c>
       <c r="I76">
-        <v>0.6839</v>
+        <v>0.6988</v>
       </c>
       <c r="J76">
-        <v>0.2313</v>
+        <v>0.2148</v>
       </c>
       <c r="K76">
-        <v>0.401</v>
+        <v>0.3876</v>
       </c>
       <c r="L76">
-        <v>0.3161</v>
+        <v>0.3012</v>
       </c>
       <c r="M76">
         <v>179</v>
@@ -4095,22 +4095,22 @@
         <v>67</v>
       </c>
       <c r="G80">
-        <v>0.7082000000000001</v>
+        <v>0.715</v>
       </c>
       <c r="H80">
-        <v>0.5289</v>
+        <v>0.5352</v>
       </c>
       <c r="I80">
-        <v>0.6186</v>
+        <v>0.6251</v>
       </c>
       <c r="J80">
-        <v>0.2918</v>
+        <v>0.285</v>
       </c>
       <c r="K80">
-        <v>0.4711</v>
+        <v>0.4648</v>
       </c>
       <c r="L80">
-        <v>0.3814</v>
+        <v>0.3749</v>
       </c>
       <c r="M80">
         <v>179</v>
@@ -4274,19 +4274,19 @@
         <v>0.5664</v>
       </c>
       <c r="H84">
-        <v>0.4245</v>
+        <v>0.4314</v>
       </c>
       <c r="I84">
-        <v>0.4954</v>
+        <v>0.4989</v>
       </c>
       <c r="J84">
         <v>0.4336</v>
       </c>
       <c r="K84">
-        <v>0.5755</v>
+        <v>0.5686</v>
       </c>
       <c r="L84">
-        <v>0.5046</v>
+        <v>0.5011</v>
       </c>
       <c r="M84">
         <v>179</v>
@@ -4318,19 +4318,19 @@
         <v>0.6738</v>
       </c>
       <c r="H85">
-        <v>0.5249</v>
+        <v>0.5254</v>
       </c>
       <c r="I85">
-        <v>0.5994</v>
+        <v>0.5996</v>
       </c>
       <c r="J85">
         <v>0.3262</v>
       </c>
       <c r="K85">
-        <v>0.4751</v>
+        <v>0.4746</v>
       </c>
       <c r="L85">
-        <v>0.4006</v>
+        <v>0.4004</v>
       </c>
       <c r="M85">
         <v>179</v>
@@ -4494,19 +4494,19 @@
         <v>0.3817</v>
       </c>
       <c r="H89">
-        <v>0.2119</v>
+        <v>0.208</v>
       </c>
       <c r="I89">
-        <v>0.2968</v>
+        <v>0.2948</v>
       </c>
       <c r="J89">
         <v>0.6183</v>
       </c>
       <c r="K89">
-        <v>0.7881</v>
+        <v>0.792</v>
       </c>
       <c r="L89">
-        <v>0.7032</v>
+        <v>0.7052</v>
       </c>
       <c r="M89">
         <v>179</v>
@@ -4887,22 +4887,22 @@
         <v>59</v>
       </c>
       <c r="G98">
-        <v>0.3505</v>
+        <v>0.3495</v>
       </c>
       <c r="H98">
-        <v>0.2181</v>
+        <v>0.2196</v>
       </c>
       <c r="I98">
-        <v>0.2843</v>
+        <v>0.2845</v>
       </c>
       <c r="J98">
-        <v>0.6495</v>
+        <v>0.6505</v>
       </c>
       <c r="K98">
-        <v>0.7819</v>
+        <v>0.7804</v>
       </c>
       <c r="L98">
-        <v>0.7157</v>
+        <v>0.7155</v>
       </c>
       <c r="M98">
         <v>179</v>
@@ -4978,19 +4978,19 @@
         <v>0.3618</v>
       </c>
       <c r="H100">
-        <v>0.198</v>
+        <v>0.1944</v>
       </c>
       <c r="I100">
-        <v>0.2799</v>
+        <v>0.2781</v>
       </c>
       <c r="J100">
         <v>0.6382</v>
       </c>
       <c r="K100">
-        <v>0.802</v>
+        <v>0.8056</v>
       </c>
       <c r="L100">
-        <v>0.7201</v>
+        <v>0.7219</v>
       </c>
       <c r="M100">
         <v>179</v>
@@ -5063,22 +5063,22 @@
         <v>63</v>
       </c>
       <c r="G102">
-        <v>0.3659</v>
+        <v>0.3751</v>
       </c>
       <c r="H102">
-        <v>0.2102</v>
+        <v>0.2259</v>
       </c>
       <c r="I102">
-        <v>0.2881</v>
+        <v>0.3005</v>
       </c>
       <c r="J102">
-        <v>0.6341</v>
+        <v>0.6249</v>
       </c>
       <c r="K102">
-        <v>0.7897999999999999</v>
+        <v>0.7741</v>
       </c>
       <c r="L102">
-        <v>0.7119</v>
+        <v>0.6995</v>
       </c>
       <c r="M102">
         <v>179</v>
@@ -5239,22 +5239,22 @@
         <v>67</v>
       </c>
       <c r="G106">
-        <v>0.2996</v>
+        <v>0.3055</v>
       </c>
       <c r="H106">
-        <v>0.148</v>
+        <v>0.1505</v>
       </c>
       <c r="I106">
-        <v>0.2238</v>
+        <v>0.228</v>
       </c>
       <c r="J106">
-        <v>0.7004</v>
+        <v>0.6945</v>
       </c>
       <c r="K106">
-        <v>0.852</v>
+        <v>0.8495</v>
       </c>
       <c r="L106">
-        <v>0.7762</v>
+        <v>0.772</v>
       </c>
       <c r="M106">
         <v>179</v>
@@ -5415,22 +5415,22 @@
         <v>71</v>
       </c>
       <c r="G110">
-        <v>0.2559</v>
+        <v>0.2522</v>
       </c>
       <c r="H110">
         <v>0.1324</v>
       </c>
       <c r="I110">
-        <v>0.1942</v>
+        <v>0.1923</v>
       </c>
       <c r="J110">
-        <v>0.7441</v>
+        <v>0.7478</v>
       </c>
       <c r="K110">
         <v>0.8676</v>
       </c>
       <c r="L110">
-        <v>0.8058</v>
+        <v>0.8077</v>
       </c>
       <c r="M110">
         <v>179</v>
@@ -5459,22 +5459,22 @@
         <v>73</v>
       </c>
       <c r="G111">
-        <v>0.2848</v>
+        <v>0.2818</v>
       </c>
       <c r="H111">
         <v>0.1603</v>
       </c>
       <c r="I111">
-        <v>0.2226</v>
+        <v>0.221</v>
       </c>
       <c r="J111">
-        <v>0.7151999999999999</v>
+        <v>0.7181999999999999</v>
       </c>
       <c r="K111">
         <v>0.8397</v>
       </c>
       <c r="L111">
-        <v>0.7774</v>
+        <v>0.779</v>
       </c>
       <c r="M111">
         <v>179</v>
@@ -5635,22 +5635,22 @@
         <v>51</v>
       </c>
       <c r="G115">
-        <v>0.3143</v>
+        <v>0.3142</v>
       </c>
       <c r="H115">
-        <v>0.1587</v>
+        <v>0.1575</v>
       </c>
       <c r="I115">
-        <v>0.2365</v>
+        <v>0.2358</v>
       </c>
       <c r="J115">
-        <v>0.6857</v>
+        <v>0.6858</v>
       </c>
       <c r="K115">
-        <v>0.8413</v>
+        <v>0.8425</v>
       </c>
       <c r="L115">
-        <v>0.7635</v>
+        <v>0.7642</v>
       </c>
       <c r="M115">
         <v>179</v>
@@ -5679,22 +5679,22 @@
         <v>52</v>
       </c>
       <c r="G116">
-        <v>0.3386</v>
+        <v>0.3455</v>
       </c>
       <c r="H116">
         <v>0.1752</v>
       </c>
       <c r="I116">
-        <v>0.2569</v>
+        <v>0.2603</v>
       </c>
       <c r="J116">
-        <v>0.6614</v>
+        <v>0.6545</v>
       </c>
       <c r="K116">
         <v>0.8248</v>
       </c>
       <c r="L116">
-        <v>0.7431</v>
+        <v>0.7397</v>
       </c>
       <c r="M116">
         <v>179</v>
@@ -5899,22 +5899,22 @@
         <v>57</v>
       </c>
       <c r="G121">
-        <v>0.7375</v>
+        <v>0.7373</v>
       </c>
       <c r="H121">
         <v>0.5495</v>
       </c>
       <c r="I121">
-        <v>0.6435</v>
+        <v>0.6434</v>
       </c>
       <c r="J121">
-        <v>0.2625</v>
+        <v>0.2627</v>
       </c>
       <c r="K121">
         <v>0.4505</v>
       </c>
       <c r="L121">
-        <v>0.3565</v>
+        <v>0.3566</v>
       </c>
       <c r="M121">
         <v>179</v>
@@ -6122,19 +6122,19 @@
         <v>0.3751</v>
       </c>
       <c r="H126">
-        <v>0.1871</v>
+        <v>0.1891</v>
       </c>
       <c r="I126">
-        <v>0.2811</v>
+        <v>0.2821</v>
       </c>
       <c r="J126">
         <v>0.6249</v>
       </c>
       <c r="K126">
-        <v>0.8129</v>
+        <v>0.8109</v>
       </c>
       <c r="L126">
-        <v>0.7189</v>
+        <v>0.7179</v>
       </c>
       <c r="M126">
         <v>179</v>
@@ -6163,22 +6163,22 @@
         <v>63</v>
       </c>
       <c r="G127">
-        <v>0.391</v>
+        <v>0.4043</v>
       </c>
       <c r="H127">
-        <v>0.2202</v>
+        <v>0.2535</v>
       </c>
       <c r="I127">
-        <v>0.3056</v>
+        <v>0.3289</v>
       </c>
       <c r="J127">
-        <v>0.609</v>
+        <v>0.5957</v>
       </c>
       <c r="K127">
-        <v>0.7798</v>
+        <v>0.7465000000000001</v>
       </c>
       <c r="L127">
-        <v>0.6944</v>
+        <v>0.6711</v>
       </c>
       <c r="M127">
         <v>179</v>
@@ -6339,22 +6339,22 @@
         <v>67</v>
       </c>
       <c r="G131">
-        <v>0.3473</v>
+        <v>0.3503</v>
       </c>
       <c r="H131">
-        <v>0.1562</v>
+        <v>0.1586</v>
       </c>
       <c r="I131">
-        <v>0.2518</v>
+        <v>0.2544</v>
       </c>
       <c r="J131">
-        <v>0.6526999999999999</v>
+        <v>0.6497000000000001</v>
       </c>
       <c r="K131">
-        <v>0.8438</v>
+        <v>0.8414</v>
       </c>
       <c r="L131">
-        <v>0.7482</v>
+        <v>0.7456</v>
       </c>
       <c r="M131">
         <v>179</v>
@@ -6738,19 +6738,19 @@
         <v>0.3174</v>
       </c>
       <c r="H140">
-        <v>0.1648</v>
+        <v>0.1714</v>
       </c>
       <c r="I140">
-        <v>0.2411</v>
+        <v>0.2444</v>
       </c>
       <c r="J140">
         <v>0.6826</v>
       </c>
       <c r="K140">
-        <v>0.8352000000000001</v>
+        <v>0.8286</v>
       </c>
       <c r="L140">
-        <v>0.7589</v>
+        <v>0.7556</v>
       </c>
       <c r="M140">
         <v>179</v>
@@ -6914,19 +6914,19 @@
         <v>0.3</v>
       </c>
       <c r="H144">
-        <v>0.1754</v>
+        <v>0.1721</v>
       </c>
       <c r="I144">
-        <v>0.2377</v>
+        <v>0.236</v>
       </c>
       <c r="J144">
         <v>0.7</v>
       </c>
       <c r="K144">
-        <v>0.8246</v>
+        <v>0.8279</v>
       </c>
       <c r="L144">
-        <v>0.7623</v>
+        <v>0.764</v>
       </c>
       <c r="M144">
         <v>179</v>
@@ -7043,22 +7043,22 @@
         <v>59</v>
       </c>
       <c r="G147">
-        <v>0.3391</v>
+        <v>0.346</v>
       </c>
       <c r="H147">
-        <v>0.2005</v>
+        <v>0.2051</v>
       </c>
       <c r="I147">
-        <v>0.2698</v>
+        <v>0.2755</v>
       </c>
       <c r="J147">
-        <v>0.6609</v>
+        <v>0.654</v>
       </c>
       <c r="K147">
-        <v>0.7995</v>
+        <v>0.7949000000000001</v>
       </c>
       <c r="L147">
-        <v>0.7302</v>
+        <v>0.7245</v>
       </c>
       <c r="M147">
         <v>179</v>
@@ -7175,22 +7175,22 @@
         <v>62</v>
       </c>
       <c r="G150">
-        <v>0.3318</v>
+        <v>0.3309</v>
       </c>
       <c r="H150">
         <v>0.1867</v>
       </c>
       <c r="I150">
-        <v>0.2592</v>
+        <v>0.2588</v>
       </c>
       <c r="J150">
-        <v>0.6682</v>
+        <v>0.6691</v>
       </c>
       <c r="K150">
         <v>0.8133</v>
       </c>
       <c r="L150">
-        <v>0.7408</v>
+        <v>0.7412</v>
       </c>
       <c r="M150">
         <v>179</v>
@@ -7219,22 +7219,22 @@
         <v>63</v>
       </c>
       <c r="G151">
-        <v>0.3642</v>
+        <v>0.3771</v>
       </c>
       <c r="H151">
-        <v>0.197</v>
+        <v>0.2073</v>
       </c>
       <c r="I151">
-        <v>0.2806</v>
+        <v>0.2922</v>
       </c>
       <c r="J151">
-        <v>0.6358</v>
+        <v>0.6229</v>
       </c>
       <c r="K151">
-        <v>0.803</v>
+        <v>0.7927</v>
       </c>
       <c r="L151">
-        <v>0.7194</v>
+        <v>0.7078</v>
       </c>
       <c r="M151">
         <v>179</v>
@@ -7310,19 +7310,19 @@
         <v>0.2577</v>
       </c>
       <c r="H153">
-        <v>0.1418</v>
+        <v>0.1396</v>
       </c>
       <c r="I153">
-        <v>0.1997</v>
+        <v>0.1986</v>
       </c>
       <c r="J153">
         <v>0.7423</v>
       </c>
       <c r="K153">
-        <v>0.8582</v>
+        <v>0.8604000000000001</v>
       </c>
       <c r="L153">
-        <v>0.8003</v>
+        <v>0.8014</v>
       </c>
       <c r="M153">
         <v>179</v>
@@ -7354,19 +7354,19 @@
         <v>0.2987</v>
       </c>
       <c r="H154">
-        <v>0.1981</v>
+        <v>0.1975</v>
       </c>
       <c r="I154">
-        <v>0.2484</v>
+        <v>0.2481</v>
       </c>
       <c r="J154">
         <v>0.7013</v>
       </c>
       <c r="K154">
-        <v>0.8018999999999999</v>
+        <v>0.8025</v>
       </c>
       <c r="L154">
-        <v>0.7516</v>
+        <v>0.7519</v>
       </c>
       <c r="M154">
         <v>179</v>
@@ -7395,22 +7395,22 @@
         <v>67</v>
       </c>
       <c r="G155">
-        <v>0.2873</v>
+        <v>0.2922</v>
       </c>
       <c r="H155">
         <v>0.1558</v>
       </c>
       <c r="I155">
-        <v>0.2216</v>
+        <v>0.224</v>
       </c>
       <c r="J155">
-        <v>0.7127</v>
+        <v>0.7078</v>
       </c>
       <c r="K155">
         <v>0.8442</v>
       </c>
       <c r="L155">
-        <v>0.7784</v>
+        <v>0.776</v>
       </c>
       <c r="M155">
         <v>179</v>
@@ -7703,22 +7703,22 @@
         <v>51</v>
       </c>
       <c r="G162">
-        <v>0.6807</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="H162">
         <v>0.5163</v>
       </c>
       <c r="I162">
-        <v>0.5985</v>
+        <v>0.5992</v>
       </c>
       <c r="J162">
-        <v>0.3193</v>
+        <v>0.318</v>
       </c>
       <c r="K162">
         <v>0.4837</v>
       </c>
       <c r="L162">
-        <v>0.4015</v>
+        <v>0.4008</v>
       </c>
       <c r="M162">
         <v>179</v>
@@ -7750,19 +7750,19 @@
         <v>0.7305</v>
       </c>
       <c r="H163">
-        <v>0.5647</v>
+        <v>0.5686</v>
       </c>
       <c r="I163">
-        <v>0.6476</v>
+        <v>0.6496</v>
       </c>
       <c r="J163">
         <v>0.2695</v>
       </c>
       <c r="K163">
-        <v>0.4353</v>
+        <v>0.4314</v>
       </c>
       <c r="L163">
-        <v>0.3524</v>
+        <v>0.3504</v>
       </c>
       <c r="M163">
         <v>179</v>
@@ -7835,22 +7835,22 @@
         <v>54</v>
       </c>
       <c r="G165">
-        <v>0.7798</v>
+        <v>0.7811</v>
       </c>
       <c r="H165">
         <v>0.5772</v>
       </c>
       <c r="I165">
-        <v>0.6785</v>
+        <v>0.6792</v>
       </c>
       <c r="J165">
-        <v>0.2202</v>
+        <v>0.2189</v>
       </c>
       <c r="K165">
         <v>0.4228</v>
       </c>
       <c r="L165">
-        <v>0.3215</v>
+        <v>0.3208</v>
       </c>
       <c r="M165">
         <v>179</v>
@@ -7926,19 +7926,19 @@
         <v>0.7055</v>
       </c>
       <c r="H167">
-        <v>0.573</v>
+        <v>0.5783</v>
       </c>
       <c r="I167">
-        <v>0.6392</v>
+        <v>0.6419</v>
       </c>
       <c r="J167">
         <v>0.2945</v>
       </c>
       <c r="K167">
-        <v>0.427</v>
+        <v>0.4217</v>
       </c>
       <c r="L167">
-        <v>0.3608</v>
+        <v>0.3581</v>
       </c>
       <c r="M167">
         <v>179</v>
@@ -8055,22 +8055,22 @@
         <v>59</v>
       </c>
       <c r="G170">
-        <v>0.7858000000000001</v>
+        <v>0.787</v>
       </c>
       <c r="H170">
-        <v>0.6113</v>
+        <v>0.6136</v>
       </c>
       <c r="I170">
-        <v>0.6986</v>
+        <v>0.7003</v>
       </c>
       <c r="J170">
-        <v>0.2142</v>
+        <v>0.213</v>
       </c>
       <c r="K170">
-        <v>0.3887</v>
+        <v>0.3864</v>
       </c>
       <c r="L170">
-        <v>0.3014</v>
+        <v>0.2997</v>
       </c>
       <c r="M170">
         <v>179</v>
@@ -8187,22 +8187,22 @@
         <v>62</v>
       </c>
       <c r="G173">
-        <v>0.7423999999999999</v>
+        <v>0.7438</v>
       </c>
       <c r="H173">
         <v>0.5921999999999999</v>
       </c>
       <c r="I173">
-        <v>0.6673</v>
+        <v>0.668</v>
       </c>
       <c r="J173">
-        <v>0.2576</v>
+        <v>0.2562</v>
       </c>
       <c r="K173">
         <v>0.4078</v>
       </c>
       <c r="L173">
-        <v>0.3327</v>
+        <v>0.332</v>
       </c>
       <c r="M173">
         <v>179</v>
@@ -8231,22 +8231,22 @@
         <v>63</v>
       </c>
       <c r="G174">
-        <v>0.7735</v>
+        <v>0.7883</v>
       </c>
       <c r="H174">
-        <v>0.5846</v>
+        <v>0.598</v>
       </c>
       <c r="I174">
-        <v>0.679</v>
+        <v>0.6931</v>
       </c>
       <c r="J174">
-        <v>0.2265</v>
+        <v>0.2117</v>
       </c>
       <c r="K174">
-        <v>0.4154</v>
+        <v>0.402</v>
       </c>
       <c r="L174">
-        <v>0.321</v>
+        <v>0.3069</v>
       </c>
       <c r="M174">
         <v>179</v>
@@ -8407,22 +8407,22 @@
         <v>67</v>
       </c>
       <c r="G178">
-        <v>0.7010999999999999</v>
+        <v>0.7135</v>
       </c>
       <c r="H178">
-        <v>0.5574</v>
+        <v>0.5636</v>
       </c>
       <c r="I178">
-        <v>0.6292</v>
+        <v>0.6385</v>
       </c>
       <c r="J178">
-        <v>0.2989</v>
+        <v>0.2865</v>
       </c>
       <c r="K178">
-        <v>0.4426</v>
+        <v>0.4364</v>
       </c>
       <c r="L178">
-        <v>0.3708</v>
+        <v>0.3615</v>
       </c>
       <c r="M178">
         <v>179</v>
@@ -8586,19 +8586,19 @@
         <v>0.624</v>
       </c>
       <c r="H182">
-        <v>0.4328</v>
+        <v>0.4397</v>
       </c>
       <c r="I182">
-        <v>0.5284</v>
+        <v>0.5318000000000001</v>
       </c>
       <c r="J182">
         <v>0.376</v>
       </c>
       <c r="K182">
-        <v>0.5672</v>
+        <v>0.5603</v>
       </c>
       <c r="L182">
-        <v>0.4716</v>
+        <v>0.4682</v>
       </c>
       <c r="M182">
         <v>179</v>
@@ -8630,19 +8630,19 @@
         <v>0.7056</v>
       </c>
       <c r="H183">
-        <v>0.5443</v>
+        <v>0.5448</v>
       </c>
       <c r="I183">
-        <v>0.625</v>
+        <v>0.6252</v>
       </c>
       <c r="J183">
         <v>0.2944</v>
       </c>
       <c r="K183">
-        <v>0.4557</v>
+        <v>0.4552</v>
       </c>
       <c r="L183">
-        <v>0.375</v>
+        <v>0.3748</v>
       </c>
       <c r="M183">
         <v>179</v>
@@ -8715,22 +8715,22 @@
         <v>52</v>
       </c>
       <c r="G185">
-        <v>0.4998</v>
+        <v>0.5091</v>
       </c>
       <c r="H185">
-        <v>0.3514</v>
+        <v>0.3525</v>
       </c>
       <c r="I185">
-        <v>0.4256</v>
+        <v>0.4308</v>
       </c>
       <c r="J185">
-        <v>0.5002</v>
+        <v>0.4909</v>
       </c>
       <c r="K185">
-        <v>0.6486</v>
+        <v>0.6475</v>
       </c>
       <c r="L185">
-        <v>0.5744</v>
+        <v>0.5692</v>
       </c>
       <c r="M185">
         <v>179</v>
@@ -8935,22 +8935,22 @@
         <v>57</v>
       </c>
       <c r="G190">
-        <v>0.8368</v>
+        <v>0.8383</v>
       </c>
       <c r="H190">
         <v>0.7257</v>
       </c>
       <c r="I190">
-        <v>0.7812</v>
+        <v>0.782</v>
       </c>
       <c r="J190">
-        <v>0.1632</v>
+        <v>0.1617</v>
       </c>
       <c r="K190">
         <v>0.2743</v>
       </c>
       <c r="L190">
-        <v>0.2188</v>
+        <v>0.218</v>
       </c>
       <c r="M190">
         <v>179</v>
@@ -9023,22 +9023,22 @@
         <v>59</v>
       </c>
       <c r="G192">
-        <v>0.577</v>
+        <v>0.5851</v>
       </c>
       <c r="H192">
         <v>0.4295</v>
       </c>
       <c r="I192">
-        <v>0.5032</v>
+        <v>0.5073</v>
       </c>
       <c r="J192">
-        <v>0.423</v>
+        <v>0.4149</v>
       </c>
       <c r="K192">
         <v>0.5705</v>
       </c>
       <c r="L192">
-        <v>0.4968</v>
+        <v>0.4927</v>
       </c>
       <c r="M192">
         <v>179</v>
@@ -9067,22 +9067,22 @@
         <v>60</v>
       </c>
       <c r="G193">
-        <v>0.7857</v>
+        <v>0.7867</v>
       </c>
       <c r="H193">
         <v>0.6098</v>
       </c>
       <c r="I193">
-        <v>0.6978</v>
+        <v>0.6982</v>
       </c>
       <c r="J193">
-        <v>0.2143</v>
+        <v>0.2133</v>
       </c>
       <c r="K193">
         <v>0.3902</v>
       </c>
       <c r="L193">
-        <v>0.3022</v>
+        <v>0.3018</v>
       </c>
       <c r="M193">
         <v>179</v>
@@ -9155,22 +9155,22 @@
         <v>62</v>
       </c>
       <c r="G195">
-        <v>0.5185999999999999</v>
+        <v>0.5377999999999999</v>
       </c>
       <c r="H195">
-        <v>0.3982</v>
+        <v>0.3998</v>
       </c>
       <c r="I195">
-        <v>0.4584</v>
+        <v>0.4688</v>
       </c>
       <c r="J195">
-        <v>0.4814</v>
+        <v>0.4622</v>
       </c>
       <c r="K195">
-        <v>0.6018</v>
+        <v>0.6002</v>
       </c>
       <c r="L195">
-        <v>0.5416</v>
+        <v>0.5312</v>
       </c>
       <c r="M195">
         <v>179</v>
@@ -9199,22 +9199,22 @@
         <v>63</v>
       </c>
       <c r="G196">
-        <v>0.5358000000000001</v>
+        <v>0.5889</v>
       </c>
       <c r="H196">
-        <v>0.4032</v>
+        <v>0.4149</v>
       </c>
       <c r="I196">
-        <v>0.4695</v>
+        <v>0.5019</v>
       </c>
       <c r="J196">
-        <v>0.4642</v>
+        <v>0.4111</v>
       </c>
       <c r="K196">
-        <v>0.5968</v>
+        <v>0.5851</v>
       </c>
       <c r="L196">
-        <v>0.5305</v>
+        <v>0.4981</v>
       </c>
       <c r="M196">
         <v>179</v>
@@ -9375,22 +9375,22 @@
         <v>67</v>
       </c>
       <c r="G200">
-        <v>0.4707</v>
+        <v>0.4848</v>
       </c>
       <c r="H200">
-        <v>0.3475</v>
+        <v>0.3553</v>
       </c>
       <c r="I200">
-        <v>0.4091</v>
+        <v>0.42</v>
       </c>
       <c r="J200">
-        <v>0.5293</v>
+        <v>0.5152</v>
       </c>
       <c r="K200">
-        <v>0.6525</v>
+        <v>0.6447000000000001</v>
       </c>
       <c r="L200">
-        <v>0.5909</v>
+        <v>0.58</v>
       </c>
       <c r="M200">
         <v>179</v>
@@ -9419,22 +9419,22 @@
         <v>68</v>
       </c>
       <c r="G201">
-        <v>0.7916</v>
+        <v>0.793</v>
       </c>
       <c r="H201">
         <v>0.666</v>
       </c>
       <c r="I201">
-        <v>0.7288</v>
+        <v>0.7295</v>
       </c>
       <c r="J201">
-        <v>0.2084</v>
+        <v>0.207</v>
       </c>
       <c r="K201">
         <v>0.334</v>
       </c>
       <c r="L201">
-        <v>0.2712</v>
+        <v>0.2705</v>
       </c>
       <c r="M201">
         <v>179</v>
@@ -9466,19 +9466,19 @@
         <v>0.8064</v>
       </c>
       <c r="H202">
-        <v>0.6465</v>
+        <v>0.6492</v>
       </c>
       <c r="I202">
-        <v>0.7264</v>
+        <v>0.7278</v>
       </c>
       <c r="J202">
         <v>0.1936</v>
       </c>
       <c r="K202">
-        <v>0.3535</v>
+        <v>0.3508</v>
       </c>
       <c r="L202">
-        <v>0.2736</v>
+        <v>0.2722</v>
       </c>
       <c r="M202">
         <v>179</v>
@@ -9551,22 +9551,22 @@
         <v>71</v>
       </c>
       <c r="G204">
-        <v>0.3895</v>
+        <v>0.3923</v>
       </c>
       <c r="H204">
         <v>0.2537</v>
       </c>
       <c r="I204">
-        <v>0.3216</v>
+        <v>0.323</v>
       </c>
       <c r="J204">
-        <v>0.6105</v>
+        <v>0.6077</v>
       </c>
       <c r="K204">
         <v>0.7463</v>
       </c>
       <c r="L204">
-        <v>0.6784</v>
+        <v>0.677</v>
       </c>
       <c r="M204">
         <v>179</v>
@@ -9595,22 +9595,22 @@
         <v>73</v>
       </c>
       <c r="G205">
-        <v>0.4791</v>
+        <v>0.4692</v>
       </c>
       <c r="H205">
         <v>0.3254</v>
       </c>
       <c r="I205">
-        <v>0.4022</v>
+        <v>0.3973</v>
       </c>
       <c r="J205">
-        <v>0.5209</v>
+        <v>0.5308</v>
       </c>
       <c r="K205">
         <v>0.6746</v>
       </c>
       <c r="L205">
-        <v>0.5978</v>
+        <v>0.6027</v>
       </c>
       <c r="M205">
         <v>179</v>
@@ -9642,19 +9642,19 @@
         <v>0.5921</v>
       </c>
       <c r="H206">
-        <v>0.4914</v>
+        <v>0.4916</v>
       </c>
       <c r="I206">
-        <v>0.5417</v>
+        <v>0.5417999999999999</v>
       </c>
       <c r="J206">
         <v>0.4079</v>
       </c>
       <c r="K206">
-        <v>0.5086000000000001</v>
+        <v>0.5084</v>
       </c>
       <c r="L206">
-        <v>0.4583</v>
+        <v>0.4582</v>
       </c>
       <c r="M206">
         <v>179</v>
@@ -9903,22 +9903,22 @@
         <v>58</v>
       </c>
       <c r="G212">
-        <v>0.4847</v>
+        <v>0.4838</v>
       </c>
       <c r="H212">
-        <v>0.3189</v>
+        <v>0.3174</v>
       </c>
       <c r="I212">
-        <v>0.4018</v>
+        <v>0.4006</v>
       </c>
       <c r="J212">
-        <v>0.5153</v>
+        <v>0.5162</v>
       </c>
       <c r="K212">
-        <v>0.6811</v>
+        <v>0.6826</v>
       </c>
       <c r="L212">
-        <v>0.5982</v>
+        <v>0.5994</v>
       </c>
       <c r="M212">
         <v>179</v>
@@ -9947,22 +9947,22 @@
         <v>59</v>
       </c>
       <c r="G213">
-        <v>0.6724</v>
+        <v>0.6741</v>
       </c>
       <c r="H213">
         <v>0.5248</v>
       </c>
       <c r="I213">
-        <v>0.5986</v>
+        <v>0.5994</v>
       </c>
       <c r="J213">
-        <v>0.3276</v>
+        <v>0.3259</v>
       </c>
       <c r="K213">
         <v>0.4752</v>
       </c>
       <c r="L213">
-        <v>0.4014</v>
+        <v>0.4006</v>
       </c>
       <c r="M213">
         <v>179</v>
@@ -9991,22 +9991,22 @@
         <v>60</v>
       </c>
       <c r="G214">
-        <v>0.8193</v>
+        <v>0.8214</v>
       </c>
       <c r="H214">
-        <v>0.7112000000000001</v>
+        <v>0.711</v>
       </c>
       <c r="I214">
-        <v>0.7652</v>
+        <v>0.7662</v>
       </c>
       <c r="J214">
-        <v>0.1807</v>
+        <v>0.1786</v>
       </c>
       <c r="K214">
-        <v>0.2888</v>
+        <v>0.289</v>
       </c>
       <c r="L214">
-        <v>0.2348</v>
+        <v>0.2338</v>
       </c>
       <c r="M214">
         <v>179</v>
@@ -10123,22 +10123,22 @@
         <v>63</v>
       </c>
       <c r="G217">
-        <v>0.6643</v>
+        <v>0.6884</v>
       </c>
       <c r="H217">
-        <v>0.5159</v>
+        <v>0.555</v>
       </c>
       <c r="I217">
-        <v>0.5901</v>
+        <v>0.6217</v>
       </c>
       <c r="J217">
-        <v>0.3357</v>
+        <v>0.3116</v>
       </c>
       <c r="K217">
-        <v>0.4841</v>
+        <v>0.445</v>
       </c>
       <c r="L217">
-        <v>0.4099</v>
+        <v>0.3783</v>
       </c>
       <c r="M217">
         <v>179</v>
@@ -10258,19 +10258,19 @@
         <v>0.5673</v>
       </c>
       <c r="H220">
-        <v>0.3864</v>
+        <v>0.3876</v>
       </c>
       <c r="I220">
-        <v>0.4768</v>
+        <v>0.4774</v>
       </c>
       <c r="J220">
         <v>0.4327</v>
       </c>
       <c r="K220">
-        <v>0.6136</v>
+        <v>0.6124000000000001</v>
       </c>
       <c r="L220">
-        <v>0.5232</v>
+        <v>0.5226</v>
       </c>
       <c r="M220">
         <v>179</v>
@@ -10299,22 +10299,22 @@
         <v>67</v>
       </c>
       <c r="G221">
-        <v>0.6091</v>
+        <v>0.611</v>
       </c>
       <c r="H221">
-        <v>0.4222</v>
+        <v>0.4442</v>
       </c>
       <c r="I221">
-        <v>0.5155999999999999</v>
+        <v>0.5276</v>
       </c>
       <c r="J221">
-        <v>0.3909</v>
+        <v>0.389</v>
       </c>
       <c r="K221">
-        <v>0.5778</v>
+        <v>0.5558</v>
       </c>
       <c r="L221">
-        <v>0.4844</v>
+        <v>0.4724</v>
       </c>
       <c r="M221">
         <v>179</v>
@@ -10519,22 +10519,22 @@
         <v>73</v>
       </c>
       <c r="G226">
-        <v>0.6057</v>
+        <v>0.6037</v>
       </c>
       <c r="H226">
-        <v>0.4237</v>
+        <v>0.4141</v>
       </c>
       <c r="I226">
-        <v>0.5147</v>
+        <v>0.5089</v>
       </c>
       <c r="J226">
-        <v>0.3943</v>
+        <v>0.3963</v>
       </c>
       <c r="K226">
-        <v>0.5763</v>
+        <v>0.5859</v>
       </c>
       <c r="L226">
-        <v>0.4853</v>
+        <v>0.4911</v>
       </c>
       <c r="M226">
         <v>179</v>
@@ -10566,19 +10566,19 @@
         <v>0.5821</v>
       </c>
       <c r="H227">
-        <v>0.4478</v>
+        <v>0.4447</v>
       </c>
       <c r="I227">
-        <v>0.515</v>
+        <v>0.5134</v>
       </c>
       <c r="J227">
         <v>0.4179</v>
       </c>
       <c r="K227">
-        <v>0.5522</v>
+        <v>0.5553</v>
       </c>
       <c r="L227">
-        <v>0.485</v>
+        <v>0.4866</v>
       </c>
       <c r="M227">
         <v>179</v>
@@ -10607,22 +10607,22 @@
         <v>54</v>
       </c>
       <c r="G228">
-        <v>0.6339</v>
+        <v>0.631</v>
       </c>
       <c r="H228">
         <v>0.4799</v>
       </c>
       <c r="I228">
-        <v>0.5569</v>
+        <v>0.5554</v>
       </c>
       <c r="J228">
-        <v>0.3661</v>
+        <v>0.369</v>
       </c>
       <c r="K228">
         <v>0.5201</v>
       </c>
       <c r="L228">
-        <v>0.4431</v>
+        <v>0.4446</v>
       </c>
       <c r="M228">
         <v>179</v>
@@ -10695,22 +10695,22 @@
         <v>56</v>
       </c>
       <c r="G230">
-        <v>0.5098</v>
+        <v>0.5026</v>
       </c>
       <c r="H230">
-        <v>0.4086</v>
+        <v>0.4061</v>
       </c>
       <c r="I230">
-        <v>0.4592</v>
+        <v>0.4544</v>
       </c>
       <c r="J230">
-        <v>0.4902</v>
+        <v>0.4974</v>
       </c>
       <c r="K230">
-        <v>0.5914</v>
+        <v>0.5939</v>
       </c>
       <c r="L230">
-        <v>0.5407999999999999</v>
+        <v>0.5456</v>
       </c>
       <c r="M230">
         <v>179</v>
@@ -10786,19 +10786,19 @@
         <v>0.4105</v>
       </c>
       <c r="H232">
-        <v>0.2716</v>
+        <v>0.2665</v>
       </c>
       <c r="I232">
-        <v>0.341</v>
+        <v>0.3385</v>
       </c>
       <c r="J232">
         <v>0.5895</v>
       </c>
       <c r="K232">
-        <v>0.7284</v>
+        <v>0.7335</v>
       </c>
       <c r="L232">
-        <v>0.659</v>
+        <v>0.6615</v>
       </c>
       <c r="M232">
         <v>179</v>
@@ -10827,22 +10827,22 @@
         <v>59</v>
       </c>
       <c r="G233">
-        <v>0.6419</v>
+        <v>0.645</v>
       </c>
       <c r="H233">
         <v>0.4979</v>
       </c>
       <c r="I233">
-        <v>0.5699</v>
+        <v>0.5714</v>
       </c>
       <c r="J233">
-        <v>0.3581</v>
+        <v>0.355</v>
       </c>
       <c r="K233">
         <v>0.5021</v>
       </c>
       <c r="L233">
-        <v>0.4301</v>
+        <v>0.4286</v>
       </c>
       <c r="M233">
         <v>179</v>
@@ -10918,19 +10918,19 @@
         <v>0.6324</v>
       </c>
       <c r="H235">
-        <v>0.4829</v>
+        <v>0.4773</v>
       </c>
       <c r="I235">
-        <v>0.5576</v>
+        <v>0.5548</v>
       </c>
       <c r="J235">
         <v>0.3676</v>
       </c>
       <c r="K235">
-        <v>0.5171</v>
+        <v>0.5227000000000001</v>
       </c>
       <c r="L235">
-        <v>0.4424</v>
+        <v>0.4452</v>
       </c>
       <c r="M235">
         <v>179</v>
@@ -11003,22 +11003,22 @@
         <v>63</v>
       </c>
       <c r="G237">
-        <v>0.6508</v>
+        <v>0.6943</v>
       </c>
       <c r="H237">
-        <v>0.459</v>
+        <v>0.4685</v>
       </c>
       <c r="I237">
-        <v>0.5548999999999999</v>
+        <v>0.5814</v>
       </c>
       <c r="J237">
-        <v>0.3492</v>
+        <v>0.3057</v>
       </c>
       <c r="K237">
-        <v>0.541</v>
+        <v>0.5315</v>
       </c>
       <c r="L237">
-        <v>0.4451</v>
+        <v>0.4186</v>
       </c>
       <c r="M237">
         <v>179</v>
@@ -11091,22 +11091,22 @@
         <v>65</v>
       </c>
       <c r="G239">
-        <v>0.4534</v>
+        <v>0.4515</v>
       </c>
       <c r="H239">
-        <v>0.3044</v>
+        <v>0.2998</v>
       </c>
       <c r="I239">
-        <v>0.3789</v>
+        <v>0.3757</v>
       </c>
       <c r="J239">
-        <v>0.5466</v>
+        <v>0.5485</v>
       </c>
       <c r="K239">
-        <v>0.6956</v>
+        <v>0.7002</v>
       </c>
       <c r="L239">
-        <v>0.6211</v>
+        <v>0.6243</v>
       </c>
       <c r="M239">
         <v>179</v>
@@ -11138,19 +11138,19 @@
         <v>0.5315</v>
       </c>
       <c r="H240">
-        <v>0.3549</v>
+        <v>0.3482</v>
       </c>
       <c r="I240">
-        <v>0.4432</v>
+        <v>0.4398</v>
       </c>
       <c r="J240">
         <v>0.4685</v>
       </c>
       <c r="K240">
-        <v>0.6451</v>
+        <v>0.6518</v>
       </c>
       <c r="L240">
-        <v>0.5568</v>
+        <v>0.5602</v>
       </c>
       <c r="M240">
         <v>179</v>
@@ -11179,22 +11179,22 @@
         <v>67</v>
       </c>
       <c r="G241">
-        <v>0.5195</v>
+        <v>0.5314</v>
       </c>
       <c r="H241">
-        <v>0.419</v>
+        <v>0.4257</v>
       </c>
       <c r="I241">
-        <v>0.4692</v>
+        <v>0.4786</v>
       </c>
       <c r="J241">
-        <v>0.4805</v>
+        <v>0.4686</v>
       </c>
       <c r="K241">
-        <v>0.581</v>
+        <v>0.5743</v>
       </c>
       <c r="L241">
-        <v>0.5308</v>
+        <v>0.5214</v>
       </c>
       <c r="M241">
         <v>179</v>
@@ -11223,22 +11223,22 @@
         <v>68</v>
       </c>
       <c r="G242">
-        <v>0.8421999999999999</v>
+        <v>0.8414</v>
       </c>
       <c r="H242">
         <v>0.6971000000000001</v>
       </c>
       <c r="I242">
-        <v>0.7696</v>
+        <v>0.7692</v>
       </c>
       <c r="J242">
-        <v>0.1578</v>
+        <v>0.1586</v>
       </c>
       <c r="K242">
         <v>0.3029</v>
       </c>
       <c r="L242">
-        <v>0.2304</v>
+        <v>0.2308</v>
       </c>
       <c r="M242">
         <v>179</v>
@@ -11399,22 +11399,22 @@
         <v>73</v>
       </c>
       <c r="G246">
-        <v>0.5262</v>
+        <v>0.522</v>
       </c>
       <c r="H246">
-        <v>0.4165</v>
+        <v>0.4117</v>
       </c>
       <c r="I246">
-        <v>0.4714</v>
+        <v>0.4668</v>
       </c>
       <c r="J246">
-        <v>0.4738</v>
+        <v>0.478</v>
       </c>
       <c r="K246">
-        <v>0.5835</v>
+        <v>0.5883</v>
       </c>
       <c r="L246">
-        <v>0.5286</v>
+        <v>0.5332</v>
       </c>
       <c r="M246">
         <v>179</v>
@@ -11487,22 +11487,22 @@
         <v>55</v>
       </c>
       <c r="G248">
-        <v>0.8207</v>
+        <v>0.8228</v>
       </c>
       <c r="H248">
-        <v>0.6725</v>
+        <v>0.6754</v>
       </c>
       <c r="I248">
-        <v>0.7466</v>
+        <v>0.7491</v>
       </c>
       <c r="J248">
-        <v>0.1793</v>
+        <v>0.1772</v>
       </c>
       <c r="K248">
-        <v>0.3275</v>
+        <v>0.3246</v>
       </c>
       <c r="L248">
-        <v>0.2534</v>
+        <v>0.2509</v>
       </c>
       <c r="M248">
         <v>179</v>
@@ -11663,22 +11663,22 @@
         <v>59</v>
       </c>
       <c r="G252">
-        <v>0.5855</v>
+        <v>0.5828</v>
       </c>
       <c r="H252">
-        <v>0.48</v>
+        <v>0.4895</v>
       </c>
       <c r="I252">
-        <v>0.5328000000000001</v>
+        <v>0.5362</v>
       </c>
       <c r="J252">
-        <v>0.4145</v>
+        <v>0.4172</v>
       </c>
       <c r="K252">
-        <v>0.52</v>
+        <v>0.5105</v>
       </c>
       <c r="L252">
-        <v>0.4672</v>
+        <v>0.4638</v>
       </c>
       <c r="M252">
         <v>179</v>
@@ -11839,22 +11839,22 @@
         <v>63</v>
       </c>
       <c r="G256">
-        <v>0.6136</v>
+        <v>0.6277</v>
       </c>
       <c r="H256">
-        <v>0.4534</v>
+        <v>0.4788</v>
       </c>
       <c r="I256">
-        <v>0.5335</v>
+        <v>0.5532</v>
       </c>
       <c r="J256">
-        <v>0.3864</v>
+        <v>0.3723</v>
       </c>
       <c r="K256">
-        <v>0.5466</v>
+        <v>0.5212</v>
       </c>
       <c r="L256">
-        <v>0.4665</v>
+        <v>0.4468</v>
       </c>
       <c r="M256">
         <v>179</v>
@@ -11930,19 +11930,19 @@
         <v>0.4122</v>
       </c>
       <c r="H258">
-        <v>0.2839</v>
+        <v>0.2831</v>
       </c>
       <c r="I258">
-        <v>0.348</v>
+        <v>0.3476</v>
       </c>
       <c r="J258">
         <v>0.5878</v>
       </c>
       <c r="K258">
-        <v>0.7161</v>
+        <v>0.7169</v>
       </c>
       <c r="L258">
-        <v>0.652</v>
+        <v>0.6524</v>
       </c>
       <c r="M258">
         <v>179</v>
@@ -12018,19 +12018,19 @@
         <v>0.5318000000000001</v>
       </c>
       <c r="H260">
-        <v>0.3659</v>
+        <v>0.3943</v>
       </c>
       <c r="I260">
-        <v>0.4488</v>
+        <v>0.463</v>
       </c>
       <c r="J260">
         <v>0.4682</v>
       </c>
       <c r="K260">
-        <v>0.6341</v>
+        <v>0.6057</v>
       </c>
       <c r="L260">
-        <v>0.5512</v>
+        <v>0.537</v>
       </c>
       <c r="M260">
         <v>179</v>
@@ -12106,19 +12106,19 @@
         <v>0.8276</v>
       </c>
       <c r="H262">
-        <v>0.6839</v>
+        <v>0.6834</v>
       </c>
       <c r="I262">
-        <v>0.7557</v>
+        <v>0.7554999999999999</v>
       </c>
       <c r="J262">
         <v>0.1724</v>
       </c>
       <c r="K262">
-        <v>0.3161</v>
+        <v>0.3166</v>
       </c>
       <c r="L262">
-        <v>0.2443</v>
+        <v>0.2445</v>
       </c>
       <c r="M262">
         <v>179</v>
@@ -12238,19 +12238,19 @@
         <v>0.5231</v>
       </c>
       <c r="H265">
-        <v>0.371</v>
+        <v>0.3596</v>
       </c>
       <c r="I265">
-        <v>0.447</v>
+        <v>0.4414</v>
       </c>
       <c r="J265">
         <v>0.4769</v>
       </c>
       <c r="K265">
-        <v>0.629</v>
+        <v>0.6404</v>
       </c>
       <c r="L265">
-        <v>0.553</v>
+        <v>0.5586</v>
       </c>
       <c r="M265">
         <v>179</v>
@@ -12455,22 +12455,22 @@
         <v>59</v>
       </c>
       <c r="G270">
-        <v>0.5721000000000001</v>
+        <v>0.5747</v>
       </c>
       <c r="H270">
-        <v>0.4307</v>
+        <v>0.4414</v>
       </c>
       <c r="I270">
-        <v>0.5014</v>
+        <v>0.508</v>
       </c>
       <c r="J270">
-        <v>0.4279</v>
+        <v>0.4253</v>
       </c>
       <c r="K270">
-        <v>0.5693</v>
+        <v>0.5586</v>
       </c>
       <c r="L270">
-        <v>0.4986</v>
+        <v>0.492</v>
       </c>
       <c r="M270">
         <v>179</v>
@@ -12590,19 +12590,19 @@
         <v>0.5647</v>
       </c>
       <c r="H273">
-        <v>0.3876</v>
+        <v>0.3915</v>
       </c>
       <c r="I273">
-        <v>0.4762</v>
+        <v>0.4781</v>
       </c>
       <c r="J273">
         <v>0.4353</v>
       </c>
       <c r="K273">
-        <v>0.6124000000000001</v>
+        <v>0.6085</v>
       </c>
       <c r="L273">
-        <v>0.5238</v>
+        <v>0.5219</v>
       </c>
       <c r="M273">
         <v>179</v>
@@ -12631,22 +12631,22 @@
         <v>63</v>
       </c>
       <c r="G274">
-        <v>0.5845</v>
+        <v>0.6038</v>
       </c>
       <c r="H274">
-        <v>0.4271</v>
+        <v>0.4477</v>
       </c>
       <c r="I274">
-        <v>0.5058</v>
+        <v>0.5256999999999999</v>
       </c>
       <c r="J274">
-        <v>0.4155</v>
+        <v>0.3962</v>
       </c>
       <c r="K274">
-        <v>0.5729</v>
+        <v>0.5523</v>
       </c>
       <c r="L274">
-        <v>0.4942</v>
+        <v>0.4743</v>
       </c>
       <c r="M274">
         <v>179</v>
@@ -12807,22 +12807,22 @@
         <v>67</v>
       </c>
       <c r="G278">
-        <v>0.5143</v>
+        <v>0.5195</v>
       </c>
       <c r="H278">
-        <v>0.3437</v>
+        <v>0.3551</v>
       </c>
       <c r="I278">
-        <v>0.429</v>
+        <v>0.4373</v>
       </c>
       <c r="J278">
-        <v>0.4857</v>
+        <v>0.4805</v>
       </c>
       <c r="K278">
-        <v>0.6563</v>
+        <v>0.6449</v>
       </c>
       <c r="L278">
-        <v>0.571</v>
+        <v>0.5627</v>
       </c>
       <c r="M278">
         <v>179</v>
@@ -13203,22 +13203,22 @@
         <v>59</v>
       </c>
       <c r="G287">
-        <v>0.3876</v>
+        <v>0.3907</v>
       </c>
       <c r="H287">
-        <v>0.2152</v>
+        <v>0.2177</v>
       </c>
       <c r="I287">
-        <v>0.3014</v>
+        <v>0.3042</v>
       </c>
       <c r="J287">
-        <v>0.6124000000000001</v>
+        <v>0.6093</v>
       </c>
       <c r="K287">
-        <v>0.7848000000000001</v>
+        <v>0.7823</v>
       </c>
       <c r="L287">
-        <v>0.6986</v>
+        <v>0.6958</v>
       </c>
       <c r="M287">
         <v>179</v>
@@ -13379,22 +13379,22 @@
         <v>63</v>
       </c>
       <c r="G291">
-        <v>0.3652</v>
+        <v>0.3773</v>
       </c>
       <c r="H291">
-        <v>0.2178</v>
+        <v>0.2336</v>
       </c>
       <c r="I291">
-        <v>0.2915</v>
+        <v>0.3054</v>
       </c>
       <c r="J291">
-        <v>0.6348</v>
+        <v>0.6227</v>
       </c>
       <c r="K291">
-        <v>0.7822</v>
+        <v>0.7664</v>
       </c>
       <c r="L291">
-        <v>0.7085</v>
+        <v>0.6946</v>
       </c>
       <c r="M291">
         <v>179</v>
@@ -13555,22 +13555,22 @@
         <v>67</v>
       </c>
       <c r="G295">
-        <v>0.3261</v>
+        <v>0.3303</v>
       </c>
       <c r="H295">
-        <v>0.1634</v>
+        <v>0.1667</v>
       </c>
       <c r="I295">
-        <v>0.2448</v>
+        <v>0.2485</v>
       </c>
       <c r="J295">
-        <v>0.6739000000000001</v>
+        <v>0.6697</v>
       </c>
       <c r="K295">
-        <v>0.8366</v>
+        <v>0.8333</v>
       </c>
       <c r="L295">
-        <v>0.7552</v>
+        <v>0.7514999999999999</v>
       </c>
       <c r="M295">
         <v>179</v>
@@ -13866,19 +13866,19 @@
         <v>0.4421</v>
       </c>
       <c r="H302">
-        <v>0.2929</v>
+        <v>0.2914</v>
       </c>
       <c r="I302">
-        <v>0.3675</v>
+        <v>0.3668</v>
       </c>
       <c r="J302">
         <v>0.5579</v>
       </c>
       <c r="K302">
-        <v>0.7071</v>
+        <v>0.7086</v>
       </c>
       <c r="L302">
-        <v>0.6325</v>
+        <v>0.6332</v>
       </c>
       <c r="M302">
         <v>179</v>
@@ -13907,22 +13907,22 @@
         <v>59</v>
       </c>
       <c r="G303">
-        <v>0.6473</v>
+        <v>0.6623</v>
       </c>
       <c r="H303">
-        <v>0.506</v>
+        <v>0.508</v>
       </c>
       <c r="I303">
-        <v>0.5766</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="J303">
-        <v>0.3527</v>
+        <v>0.3377</v>
       </c>
       <c r="K303">
-        <v>0.494</v>
+        <v>0.492</v>
       </c>
       <c r="L303">
-        <v>0.4234</v>
+        <v>0.4148</v>
       </c>
       <c r="M303">
         <v>179</v>
@@ -14083,22 +14083,22 @@
         <v>63</v>
       </c>
       <c r="G307">
-        <v>0.6354</v>
+        <v>0.6797</v>
       </c>
       <c r="H307">
-        <v>0.486</v>
+        <v>0.4898</v>
       </c>
       <c r="I307">
-        <v>0.5607</v>
+        <v>0.5848</v>
       </c>
       <c r="J307">
-        <v>0.3646</v>
+        <v>0.3203</v>
       </c>
       <c r="K307">
-        <v>0.514</v>
+        <v>0.5102</v>
       </c>
       <c r="L307">
-        <v>0.4393</v>
+        <v>0.4152</v>
       </c>
       <c r="M307">
         <v>179</v>
@@ -14259,22 +14259,22 @@
         <v>67</v>
       </c>
       <c r="G311">
-        <v>0.5624</v>
+        <v>0.5715</v>
       </c>
       <c r="H311">
-        <v>0.4249</v>
+        <v>0.4268</v>
       </c>
       <c r="I311">
-        <v>0.4936</v>
+        <v>0.4992</v>
       </c>
       <c r="J311">
-        <v>0.4376</v>
+        <v>0.4285</v>
       </c>
       <c r="K311">
-        <v>0.5750999999999999</v>
+        <v>0.5732</v>
       </c>
       <c r="L311">
-        <v>0.5064</v>
+        <v>0.5008</v>
       </c>
       <c r="M311">
         <v>179</v>
@@ -14347,22 +14347,22 @@
         <v>69</v>
       </c>
       <c r="G313">
-        <v>0.8411999999999999</v>
+        <v>0.8423</v>
       </c>
       <c r="H313">
         <v>0.7027</v>
       </c>
       <c r="I313">
-        <v>0.7719</v>
+        <v>0.7725</v>
       </c>
       <c r="J313">
-        <v>0.1588</v>
+        <v>0.1577</v>
       </c>
       <c r="K313">
         <v>0.2973</v>
       </c>
       <c r="L313">
-        <v>0.2281</v>
+        <v>0.2275</v>
       </c>
       <c r="M313">
         <v>179</v>
@@ -14567,22 +14567,22 @@
         <v>59</v>
       </c>
       <c r="G318">
-        <v>0.276</v>
+        <v>0.2787</v>
       </c>
       <c r="H318">
-        <v>0.1556</v>
+        <v>0.1582</v>
       </c>
       <c r="I318">
-        <v>0.2158</v>
+        <v>0.2184</v>
       </c>
       <c r="J318">
-        <v>0.724</v>
+        <v>0.7213000000000001</v>
       </c>
       <c r="K318">
-        <v>0.8444</v>
+        <v>0.8418</v>
       </c>
       <c r="L318">
-        <v>0.7842</v>
+        <v>0.7816</v>
       </c>
       <c r="M318">
         <v>179</v>
@@ -14743,22 +14743,22 @@
         <v>63</v>
       </c>
       <c r="G322">
-        <v>0.2768</v>
+        <v>0.2883</v>
       </c>
       <c r="H322">
-        <v>0.1405</v>
+        <v>0.1435</v>
       </c>
       <c r="I322">
-        <v>0.2086</v>
+        <v>0.2159</v>
       </c>
       <c r="J322">
-        <v>0.7232</v>
+        <v>0.7117</v>
       </c>
       <c r="K322">
-        <v>0.8595</v>
+        <v>0.8565</v>
       </c>
       <c r="L322">
-        <v>0.7914</v>
+        <v>0.7841</v>
       </c>
       <c r="M322">
         <v>179</v>
@@ -14919,22 +14919,22 @@
         <v>67</v>
       </c>
       <c r="G326">
-        <v>0.2252</v>
+        <v>0.2349</v>
       </c>
       <c r="H326">
-        <v>0.1323</v>
+        <v>0.1346</v>
       </c>
       <c r="I326">
-        <v>0.1788</v>
+        <v>0.1848</v>
       </c>
       <c r="J326">
-        <v>0.7748</v>
+        <v>0.7651</v>
       </c>
       <c r="K326">
-        <v>0.8677</v>
+        <v>0.8653999999999999</v>
       </c>
       <c r="L326">
-        <v>0.8212</v>
+        <v>0.8152</v>
       </c>
       <c r="M326">
         <v>179</v>
@@ -15142,19 +15142,19 @@
         <v>0.2183</v>
       </c>
       <c r="H331">
-        <v>0.1285</v>
+        <v>0.1263</v>
       </c>
       <c r="I331">
-        <v>0.1734</v>
+        <v>0.1723</v>
       </c>
       <c r="J331">
         <v>0.7817</v>
       </c>
       <c r="K331">
-        <v>0.8715000000000001</v>
+        <v>0.8737</v>
       </c>
       <c r="L331">
-        <v>0.8266</v>
+        <v>0.8277</v>
       </c>
       <c r="M331">
         <v>179</v>
@@ -15183,22 +15183,22 @@
         <v>59</v>
       </c>
       <c r="G332">
-        <v>0.7783</v>
+        <v>0.7808</v>
       </c>
       <c r="H332">
-        <v>0.6195000000000001</v>
+        <v>0.6238</v>
       </c>
       <c r="I332">
-        <v>0.6989</v>
+        <v>0.7023</v>
       </c>
       <c r="J332">
-        <v>0.2217</v>
+        <v>0.2192</v>
       </c>
       <c r="K332">
-        <v>0.3805</v>
+        <v>0.3762</v>
       </c>
       <c r="L332">
-        <v>0.3011</v>
+        <v>0.2977</v>
       </c>
       <c r="M332">
         <v>179</v>
@@ -15359,22 +15359,22 @@
         <v>63</v>
       </c>
       <c r="G336">
-        <v>0.7768</v>
+        <v>0.7906</v>
       </c>
       <c r="H336">
-        <v>0.6126</v>
+        <v>0.6286</v>
       </c>
       <c r="I336">
-        <v>0.6947</v>
+        <v>0.7096</v>
       </c>
       <c r="J336">
-        <v>0.2232</v>
+        <v>0.2094</v>
       </c>
       <c r="K336">
-        <v>0.3874</v>
+        <v>0.3714</v>
       </c>
       <c r="L336">
-        <v>0.3053</v>
+        <v>0.2904</v>
       </c>
       <c r="M336">
         <v>179</v>
@@ -15535,22 +15535,22 @@
         <v>67</v>
       </c>
       <c r="G340">
-        <v>0.7058</v>
+        <v>0.7181999999999999</v>
       </c>
       <c r="H340">
-        <v>0.5423</v>
+        <v>0.5668</v>
       </c>
       <c r="I340">
-        <v>0.624</v>
+        <v>0.6425</v>
       </c>
       <c r="J340">
-        <v>0.2942</v>
+        <v>0.2818</v>
       </c>
       <c r="K340">
-        <v>0.4577</v>
+        <v>0.4332</v>
       </c>
       <c r="L340">
-        <v>0.376</v>
+        <v>0.3575</v>
       </c>
       <c r="M340">
         <v>179</v>
@@ -15579,22 +15579,22 @@
         <v>68</v>
       </c>
       <c r="G341">
-        <v>0.8898</v>
+        <v>0.8928</v>
       </c>
       <c r="H341">
         <v>0.7762</v>
       </c>
       <c r="I341">
-        <v>0.833</v>
+        <v>0.8345</v>
       </c>
       <c r="J341">
-        <v>0.1102</v>
+        <v>0.1072</v>
       </c>
       <c r="K341">
         <v>0.2238</v>
       </c>
       <c r="L341">
-        <v>0.167</v>
+        <v>0.1655</v>
       </c>
       <c r="M341">
         <v>179</v>
@@ -15755,22 +15755,22 @@
         <v>73</v>
       </c>
       <c r="G345">
-        <v>0.6871</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="H345">
-        <v>0.531</v>
+        <v>0.5304</v>
       </c>
       <c r="I345">
-        <v>0.6091</v>
+        <v>0.6072</v>
       </c>
       <c r="J345">
-        <v>0.3129</v>
+        <v>0.316</v>
       </c>
       <c r="K345">
-        <v>0.469</v>
+        <v>0.4696</v>
       </c>
       <c r="L345">
-        <v>0.3909</v>
+        <v>0.3928</v>
       </c>
       <c r="M345">
         <v>179</v>
@@ -15799,22 +15799,22 @@
         <v>60</v>
       </c>
       <c r="G346">
-        <v>0.7704</v>
+        <v>0.7678</v>
       </c>
       <c r="H346">
-        <v>0.6178</v>
+        <v>0.6151</v>
       </c>
       <c r="I346">
-        <v>0.6941000000000001</v>
+        <v>0.6914</v>
       </c>
       <c r="J346">
-        <v>0.2296</v>
+        <v>0.2322</v>
       </c>
       <c r="K346">
-        <v>0.3822</v>
+        <v>0.3849</v>
       </c>
       <c r="L346">
-        <v>0.3059</v>
+        <v>0.3086</v>
       </c>
       <c r="M346">
         <v>179</v>
@@ -15843,22 +15843,22 @@
         <v>61</v>
       </c>
       <c r="G347">
-        <v>0.5612</v>
+        <v>0.5589</v>
       </c>
       <c r="H347">
-        <v>0.4526</v>
+        <v>0.4458</v>
       </c>
       <c r="I347">
-        <v>0.5069</v>
+        <v>0.5024</v>
       </c>
       <c r="J347">
-        <v>0.4388</v>
+        <v>0.4411</v>
       </c>
       <c r="K347">
-        <v>0.5474</v>
+        <v>0.5542</v>
       </c>
       <c r="L347">
-        <v>0.4931</v>
+        <v>0.4976</v>
       </c>
       <c r="M347">
         <v>179</v>
@@ -15887,22 +15887,22 @@
         <v>62</v>
       </c>
       <c r="G348">
-        <v>0.5373</v>
+        <v>0.5329</v>
       </c>
       <c r="H348">
-        <v>0.4401</v>
+        <v>0.4375</v>
       </c>
       <c r="I348">
-        <v>0.4887</v>
+        <v>0.4852</v>
       </c>
       <c r="J348">
-        <v>0.4627</v>
+        <v>0.4671</v>
       </c>
       <c r="K348">
-        <v>0.5599</v>
+        <v>0.5625</v>
       </c>
       <c r="L348">
-        <v>0.5113</v>
+        <v>0.5148</v>
       </c>
       <c r="M348">
         <v>179</v>
@@ -15931,22 +15931,22 @@
         <v>63</v>
       </c>
       <c r="G349">
-        <v>0.552</v>
+        <v>0.5711000000000001</v>
       </c>
       <c r="H349">
-        <v>0.4399</v>
+        <v>0.4606</v>
       </c>
       <c r="I349">
-        <v>0.496</v>
+        <v>0.5158</v>
       </c>
       <c r="J349">
-        <v>0.448</v>
+        <v>0.4289</v>
       </c>
       <c r="K349">
-        <v>0.5601</v>
+        <v>0.5394</v>
       </c>
       <c r="L349">
-        <v>0.504</v>
+        <v>0.4842</v>
       </c>
       <c r="M349">
         <v>179</v>
@@ -15975,22 +15975,22 @@
         <v>64</v>
       </c>
       <c r="G350">
-        <v>0.8329</v>
+        <v>0.8262</v>
       </c>
       <c r="H350">
         <v>0.6833</v>
       </c>
       <c r="I350">
-        <v>0.7581</v>
+        <v>0.7548</v>
       </c>
       <c r="J350">
-        <v>0.1671</v>
+        <v>0.1738</v>
       </c>
       <c r="K350">
         <v>0.3167</v>
       </c>
       <c r="L350">
-        <v>0.2419</v>
+        <v>0.2452</v>
       </c>
       <c r="M350">
         <v>179</v>
@@ -16019,22 +16019,22 @@
         <v>65</v>
       </c>
       <c r="G351">
-        <v>0.3788</v>
+        <v>0.3749</v>
       </c>
       <c r="H351">
-        <v>0.2604</v>
+        <v>0.254</v>
       </c>
       <c r="I351">
-        <v>0.3196</v>
+        <v>0.3144</v>
       </c>
       <c r="J351">
-        <v>0.6212</v>
+        <v>0.6251</v>
       </c>
       <c r="K351">
-        <v>0.7396</v>
+        <v>0.746</v>
       </c>
       <c r="L351">
-        <v>0.6804</v>
+        <v>0.6856</v>
       </c>
       <c r="M351">
         <v>179</v>
@@ -16066,19 +16066,19 @@
         <v>0.4722</v>
       </c>
       <c r="H352">
-        <v>0.3011</v>
+        <v>0.3</v>
       </c>
       <c r="I352">
-        <v>0.3866</v>
+        <v>0.3861</v>
       </c>
       <c r="J352">
         <v>0.5278</v>
       </c>
       <c r="K352">
-        <v>0.6989</v>
+        <v>0.7</v>
       </c>
       <c r="L352">
-        <v>0.6133999999999999</v>
+        <v>0.6139</v>
       </c>
       <c r="M352">
         <v>179</v>
@@ -16110,19 +16110,19 @@
         <v>0.5004</v>
       </c>
       <c r="H353">
-        <v>0.3544</v>
+        <v>0.3582</v>
       </c>
       <c r="I353">
-        <v>0.4274</v>
+        <v>0.4293</v>
       </c>
       <c r="J353">
         <v>0.4996</v>
       </c>
       <c r="K353">
-        <v>0.6456</v>
+        <v>0.6418</v>
       </c>
       <c r="L353">
-        <v>0.5726</v>
+        <v>0.5707</v>
       </c>
       <c r="M353">
         <v>179</v>
@@ -16151,22 +16151,22 @@
         <v>68</v>
       </c>
       <c r="G354">
-        <v>0.7939000000000001</v>
+        <v>0.7858000000000001</v>
       </c>
       <c r="H354">
-        <v>0.6635</v>
+        <v>0.6583</v>
       </c>
       <c r="I354">
-        <v>0.7287</v>
+        <v>0.7221</v>
       </c>
       <c r="J354">
-        <v>0.2061</v>
+        <v>0.2142</v>
       </c>
       <c r="K354">
-        <v>0.3365</v>
+        <v>0.3417</v>
       </c>
       <c r="L354">
-        <v>0.2713</v>
+        <v>0.2779</v>
       </c>
       <c r="M354">
         <v>179</v>
@@ -16198,19 +16198,19 @@
         <v>0.8164</v>
       </c>
       <c r="H355">
-        <v>0.6504</v>
+        <v>0.6394</v>
       </c>
       <c r="I355">
-        <v>0.7334000000000001</v>
+        <v>0.7279</v>
       </c>
       <c r="J355">
         <v>0.1836</v>
       </c>
       <c r="K355">
-        <v>0.3496</v>
+        <v>0.3606</v>
       </c>
       <c r="L355">
-        <v>0.2666</v>
+        <v>0.2721</v>
       </c>
       <c r="M355">
         <v>179</v>
@@ -16242,19 +16242,19 @@
         <v>0.8247</v>
       </c>
       <c r="H356">
-        <v>0.7118</v>
+        <v>0.7055</v>
       </c>
       <c r="I356">
-        <v>0.7682</v>
+        <v>0.7651</v>
       </c>
       <c r="J356">
         <v>0.1753</v>
       </c>
       <c r="K356">
-        <v>0.2882</v>
+        <v>0.2945</v>
       </c>
       <c r="L356">
-        <v>0.2318</v>
+        <v>0.2349</v>
       </c>
       <c r="M356">
         <v>179</v>
@@ -16283,22 +16283,22 @@
         <v>71</v>
       </c>
       <c r="G357">
-        <v>0.3865</v>
+        <v>0.3861</v>
       </c>
       <c r="H357">
-        <v>0.2498</v>
+        <v>0.2374</v>
       </c>
       <c r="I357">
-        <v>0.3182</v>
+        <v>0.3117</v>
       </c>
       <c r="J357">
-        <v>0.6135</v>
+        <v>0.6139</v>
       </c>
       <c r="K357">
-        <v>0.7502</v>
+        <v>0.7625999999999999</v>
       </c>
       <c r="L357">
-        <v>0.6818</v>
+        <v>0.6883</v>
       </c>
       <c r="M357">
         <v>179</v>
@@ -16327,22 +16327,22 @@
         <v>73</v>
       </c>
       <c r="G358">
-        <v>0.4904</v>
+        <v>0.4848</v>
       </c>
       <c r="H358">
-        <v>0.3147</v>
+        <v>0.3109</v>
       </c>
       <c r="I358">
-        <v>0.4025</v>
+        <v>0.3979</v>
       </c>
       <c r="J358">
-        <v>0.5096000000000001</v>
+        <v>0.5152</v>
       </c>
       <c r="K358">
-        <v>0.6853</v>
+        <v>0.6891</v>
       </c>
       <c r="L358">
-        <v>0.5975</v>
+        <v>0.6021</v>
       </c>
       <c r="M358">
         <v>179</v>
@@ -16374,19 +16374,19 @@
         <v>0.381</v>
       </c>
       <c r="H359">
-        <v>0.2201</v>
+        <v>0.2194</v>
       </c>
       <c r="I359">
-        <v>0.3006</v>
+        <v>0.3002</v>
       </c>
       <c r="J359">
         <v>0.619</v>
       </c>
       <c r="K359">
-        <v>0.7799</v>
+        <v>0.7806</v>
       </c>
       <c r="L359">
-        <v>0.6994</v>
+        <v>0.6998</v>
       </c>
       <c r="M359">
         <v>179</v>
@@ -16459,22 +16459,22 @@
         <v>63</v>
       </c>
       <c r="G361">
-        <v>0.3581</v>
+        <v>0.3887</v>
       </c>
       <c r="H361">
-        <v>0.2064</v>
+        <v>0.2223</v>
       </c>
       <c r="I361">
-        <v>0.2822</v>
+        <v>0.3055</v>
       </c>
       <c r="J361">
-        <v>0.6419</v>
+        <v>0.6113</v>
       </c>
       <c r="K361">
-        <v>0.7936</v>
+        <v>0.7776999999999999</v>
       </c>
       <c r="L361">
-        <v>0.7178</v>
+        <v>0.6945</v>
       </c>
       <c r="M361">
         <v>179</v>
@@ -16635,22 +16635,22 @@
         <v>67</v>
       </c>
       <c r="G365">
-        <v>0.2997</v>
+        <v>0.3037</v>
       </c>
       <c r="H365">
-        <v>0.1884</v>
+        <v>0.1908</v>
       </c>
       <c r="I365">
-        <v>0.244</v>
+        <v>0.2473</v>
       </c>
       <c r="J365">
-        <v>0.7003</v>
+        <v>0.6963</v>
       </c>
       <c r="K365">
-        <v>0.8116</v>
+        <v>0.8092</v>
       </c>
       <c r="L365">
-        <v>0.756</v>
+        <v>0.7527</v>
       </c>
       <c r="M365">
         <v>179</v>
@@ -16855,22 +16855,22 @@
         <v>73</v>
       </c>
       <c r="G370">
-        <v>0.3172</v>
+        <v>0.3126</v>
       </c>
       <c r="H370">
-        <v>0.1974</v>
+        <v>0.196</v>
       </c>
       <c r="I370">
-        <v>0.2573</v>
+        <v>0.2543</v>
       </c>
       <c r="J370">
-        <v>0.6828</v>
+        <v>0.6874</v>
       </c>
       <c r="K370">
-        <v>0.8026</v>
+        <v>0.804</v>
       </c>
       <c r="L370">
-        <v>0.7427</v>
+        <v>0.7457</v>
       </c>
       <c r="M370">
         <v>179</v>
@@ -16943,22 +16943,22 @@
         <v>63</v>
       </c>
       <c r="G372">
-        <v>0.5374</v>
+        <v>0.5709</v>
       </c>
       <c r="H372">
-        <v>0.4267</v>
+        <v>0.449</v>
       </c>
       <c r="I372">
-        <v>0.482</v>
+        <v>0.51</v>
       </c>
       <c r="J372">
-        <v>0.4626</v>
+        <v>0.4291</v>
       </c>
       <c r="K372">
-        <v>0.5733</v>
+        <v>0.551</v>
       </c>
       <c r="L372">
-        <v>0.518</v>
+        <v>0.49</v>
       </c>
       <c r="M372">
         <v>179</v>
@@ -17119,22 +17119,22 @@
         <v>67</v>
       </c>
       <c r="G376">
-        <v>0.485</v>
+        <v>0.4871</v>
       </c>
       <c r="H376">
-        <v>0.3533</v>
+        <v>0.3732</v>
       </c>
       <c r="I376">
-        <v>0.4192</v>
+        <v>0.4302</v>
       </c>
       <c r="J376">
-        <v>0.515</v>
+        <v>0.5129</v>
       </c>
       <c r="K376">
-        <v>0.6467000000000001</v>
+        <v>0.6268</v>
       </c>
       <c r="L376">
-        <v>0.5808</v>
+        <v>0.5698</v>
       </c>
       <c r="M376">
         <v>179</v>
@@ -17210,19 +17210,19 @@
         <v>0.8232</v>
       </c>
       <c r="H378">
-        <v>0.6338</v>
+        <v>0.6328</v>
       </c>
       <c r="I378">
-        <v>0.7285</v>
+        <v>0.728</v>
       </c>
       <c r="J378">
         <v>0.1768</v>
       </c>
       <c r="K378">
-        <v>0.3662</v>
+        <v>0.3672</v>
       </c>
       <c r="L378">
-        <v>0.2715</v>
+        <v>0.272</v>
       </c>
       <c r="M378">
         <v>179</v>
@@ -17383,22 +17383,22 @@
         <v>63</v>
       </c>
       <c r="G382">
-        <v>0.5698</v>
+        <v>0.5914</v>
       </c>
       <c r="H382">
-        <v>0.4224</v>
+        <v>0.4456</v>
       </c>
       <c r="I382">
-        <v>0.4961</v>
+        <v>0.5185</v>
       </c>
       <c r="J382">
-        <v>0.4302</v>
+        <v>0.4086</v>
       </c>
       <c r="K382">
-        <v>0.5776</v>
+        <v>0.5544</v>
       </c>
       <c r="L382">
-        <v>0.5039</v>
+        <v>0.4815</v>
       </c>
       <c r="M382">
         <v>179</v>
@@ -17515,22 +17515,22 @@
         <v>66</v>
       </c>
       <c r="G385">
-        <v>0.5003</v>
+        <v>0.4975</v>
       </c>
       <c r="H385">
         <v>0.3294</v>
       </c>
       <c r="I385">
-        <v>0.4148</v>
+        <v>0.4134</v>
       </c>
       <c r="J385">
-        <v>0.4997</v>
+        <v>0.5024999999999999</v>
       </c>
       <c r="K385">
         <v>0.6706</v>
       </c>
       <c r="L385">
-        <v>0.5852000000000001</v>
+        <v>0.5866</v>
       </c>
       <c r="M385">
         <v>179</v>
@@ -17559,22 +17559,22 @@
         <v>67</v>
       </c>
       <c r="G386">
-        <v>0.5177</v>
+        <v>0.5198</v>
       </c>
       <c r="H386">
-        <v>0.3718</v>
+        <v>0.3872</v>
       </c>
       <c r="I386">
-        <v>0.4448</v>
+        <v>0.4535</v>
       </c>
       <c r="J386">
-        <v>0.4823</v>
+        <v>0.4802</v>
       </c>
       <c r="K386">
-        <v>0.6282</v>
+        <v>0.6128</v>
       </c>
       <c r="L386">
-        <v>0.5552</v>
+        <v>0.5465</v>
       </c>
       <c r="M386">
         <v>179</v>
@@ -17603,22 +17603,22 @@
         <v>68</v>
       </c>
       <c r="G387">
-        <v>0.8175</v>
+        <v>0.8149</v>
       </c>
       <c r="H387">
         <v>0.6685</v>
       </c>
       <c r="I387">
-        <v>0.743</v>
+        <v>0.7417</v>
       </c>
       <c r="J387">
-        <v>0.1825</v>
+        <v>0.1851</v>
       </c>
       <c r="K387">
         <v>0.3315</v>
       </c>
       <c r="L387">
-        <v>0.257</v>
+        <v>0.2583</v>
       </c>
       <c r="M387">
         <v>179</v>
@@ -17647,22 +17647,22 @@
         <v>69</v>
       </c>
       <c r="G388">
-        <v>0.8378</v>
+        <v>0.8373</v>
       </c>
       <c r="H388">
         <v>0.6661</v>
       </c>
       <c r="I388">
-        <v>0.752</v>
+        <v>0.7517</v>
       </c>
       <c r="J388">
-        <v>0.1622</v>
+        <v>0.1627</v>
       </c>
       <c r="K388">
         <v>0.3339</v>
       </c>
       <c r="L388">
-        <v>0.248</v>
+        <v>0.2483</v>
       </c>
       <c r="M388">
         <v>179</v>
@@ -17738,19 +17738,19 @@
         <v>0.3995</v>
       </c>
       <c r="H390">
-        <v>0.2644</v>
+        <v>0.262</v>
       </c>
       <c r="I390">
-        <v>0.332</v>
+        <v>0.3308</v>
       </c>
       <c r="J390">
         <v>0.6005</v>
       </c>
       <c r="K390">
-        <v>0.7356</v>
+        <v>0.738</v>
       </c>
       <c r="L390">
-        <v>0.668</v>
+        <v>0.6692</v>
       </c>
       <c r="M390">
         <v>179</v>
@@ -17823,22 +17823,22 @@
         <v>64</v>
       </c>
       <c r="G392">
-        <v>0.8233</v>
+        <v>0.8138</v>
       </c>
       <c r="H392">
-        <v>0.696</v>
+        <v>0.6754</v>
       </c>
       <c r="I392">
-        <v>0.7596000000000001</v>
+        <v>0.7446</v>
       </c>
       <c r="J392">
-        <v>0.1767</v>
+        <v>0.1862</v>
       </c>
       <c r="K392">
-        <v>0.304</v>
+        <v>0.3246</v>
       </c>
       <c r="L392">
-        <v>0.2404</v>
+        <v>0.2554</v>
       </c>
       <c r="M392">
         <v>179</v>
@@ -17867,22 +17867,22 @@
         <v>65</v>
       </c>
       <c r="G393">
-        <v>0.3709</v>
+        <v>0.3296</v>
       </c>
       <c r="H393">
-        <v>0.3064</v>
+        <v>0.2725</v>
       </c>
       <c r="I393">
-        <v>0.3386</v>
+        <v>0.3011</v>
       </c>
       <c r="J393">
-        <v>0.6291</v>
+        <v>0.6704</v>
       </c>
       <c r="K393">
-        <v>0.6936</v>
+        <v>0.7275</v>
       </c>
       <c r="L393">
-        <v>0.6614</v>
+        <v>0.6989</v>
       </c>
       <c r="M393">
         <v>179</v>
@@ -17911,22 +17911,22 @@
         <v>66</v>
       </c>
       <c r="G394">
-        <v>0.446</v>
+        <v>0.4232</v>
       </c>
       <c r="H394">
-        <v>0.3702</v>
+        <v>0.3544</v>
       </c>
       <c r="I394">
-        <v>0.4081</v>
+        <v>0.3888</v>
       </c>
       <c r="J394">
-        <v>0.554</v>
+        <v>0.5768</v>
       </c>
       <c r="K394">
-        <v>0.6298</v>
+        <v>0.6456</v>
       </c>
       <c r="L394">
-        <v>0.5919</v>
+        <v>0.6112</v>
       </c>
       <c r="M394">
         <v>179</v>
@@ -17955,22 +17955,22 @@
         <v>67</v>
       </c>
       <c r="G395">
-        <v>0.5083</v>
+        <v>0.508</v>
       </c>
       <c r="H395">
-        <v>0.3532</v>
+        <v>0.3392</v>
       </c>
       <c r="I395">
-        <v>0.4308</v>
+        <v>0.4236</v>
       </c>
       <c r="J395">
-        <v>0.4917</v>
+        <v>0.492</v>
       </c>
       <c r="K395">
-        <v>0.6468</v>
+        <v>0.6608000000000001</v>
       </c>
       <c r="L395">
-        <v>0.5692</v>
+        <v>0.5764</v>
       </c>
       <c r="M395">
         <v>179</v>
@@ -17999,22 +17999,22 @@
         <v>68</v>
       </c>
       <c r="G396">
-        <v>0.7963</v>
+        <v>0.7869</v>
       </c>
       <c r="H396">
-        <v>0.6891</v>
+        <v>0.6643</v>
       </c>
       <c r="I396">
-        <v>0.7427</v>
+        <v>0.7256</v>
       </c>
       <c r="J396">
-        <v>0.2037</v>
+        <v>0.2131</v>
       </c>
       <c r="K396">
-        <v>0.3109</v>
+        <v>0.3357</v>
       </c>
       <c r="L396">
-        <v>0.2573</v>
+        <v>0.2744</v>
       </c>
       <c r="M396">
         <v>179</v>
@@ -18043,22 +18043,22 @@
         <v>69</v>
       </c>
       <c r="G397">
-        <v>0.7987</v>
+        <v>0.7892</v>
       </c>
       <c r="H397">
-        <v>0.6474</v>
+        <v>0.6254</v>
       </c>
       <c r="I397">
-        <v>0.723</v>
+        <v>0.7073</v>
       </c>
       <c r="J397">
-        <v>0.2013</v>
+        <v>0.2108</v>
       </c>
       <c r="K397">
-        <v>0.3526</v>
+        <v>0.3746</v>
       </c>
       <c r="L397">
-        <v>0.277</v>
+        <v>0.2927</v>
       </c>
       <c r="M397">
         <v>179</v>
@@ -18087,22 +18087,22 @@
         <v>70</v>
       </c>
       <c r="G398">
-        <v>0.8401</v>
+        <v>0.8299</v>
       </c>
       <c r="H398">
-        <v>0.7107</v>
+        <v>0.6977</v>
       </c>
       <c r="I398">
-        <v>0.7754</v>
+        <v>0.7638</v>
       </c>
       <c r="J398">
-        <v>0.1599</v>
+        <v>0.1701</v>
       </c>
       <c r="K398">
-        <v>0.2893</v>
+        <v>0.3023</v>
       </c>
       <c r="L398">
-        <v>0.2246</v>
+        <v>0.2362</v>
       </c>
       <c r="M398">
         <v>179</v>
@@ -18131,22 +18131,22 @@
         <v>71</v>
       </c>
       <c r="G399">
-        <v>0.3917</v>
+        <v>0.3814</v>
       </c>
       <c r="H399">
-        <v>0.2746</v>
+        <v>0.2408</v>
       </c>
       <c r="I399">
-        <v>0.3332</v>
+        <v>0.3111</v>
       </c>
       <c r="J399">
-        <v>0.6083</v>
+        <v>0.6186</v>
       </c>
       <c r="K399">
-        <v>0.7254</v>
+        <v>0.7592</v>
       </c>
       <c r="L399">
-        <v>0.6667999999999999</v>
+        <v>0.6889</v>
       </c>
       <c r="M399">
         <v>179</v>
@@ -18175,22 +18175,22 @@
         <v>73</v>
       </c>
       <c r="G400">
-        <v>0.5203</v>
+        <v>0.4984</v>
       </c>
       <c r="H400">
-        <v>0.307</v>
+        <v>0.2836</v>
       </c>
       <c r="I400">
-        <v>0.4136</v>
+        <v>0.391</v>
       </c>
       <c r="J400">
-        <v>0.4797</v>
+        <v>0.5016</v>
       </c>
       <c r="K400">
-        <v>0.6929999999999999</v>
+        <v>0.7164</v>
       </c>
       <c r="L400">
-        <v>0.5864</v>
+        <v>0.609</v>
       </c>
       <c r="M400">
         <v>179</v>
@@ -18310,19 +18310,19 @@
         <v>0.2675</v>
       </c>
       <c r="H403">
-        <v>0.1303</v>
+        <v>0.1352</v>
       </c>
       <c r="I403">
-        <v>0.1989</v>
+        <v>0.2014</v>
       </c>
       <c r="J403">
         <v>0.7325</v>
       </c>
       <c r="K403">
-        <v>0.8697</v>
+        <v>0.8648</v>
       </c>
       <c r="L403">
-        <v>0.8011</v>
+        <v>0.7986</v>
       </c>
       <c r="M403">
         <v>179</v>
@@ -18530,19 +18530,19 @@
         <v>0.2254</v>
       </c>
       <c r="H408">
-        <v>0.1402</v>
+        <v>0.1388</v>
       </c>
       <c r="I408">
-        <v>0.1828</v>
+        <v>0.1821</v>
       </c>
       <c r="J408">
         <v>0.7746</v>
       </c>
       <c r="K408">
-        <v>0.8598</v>
+        <v>0.8612</v>
       </c>
       <c r="L408">
-        <v>0.8172</v>
+        <v>0.8179</v>
       </c>
       <c r="M408">
         <v>179</v>
@@ -18615,22 +18615,22 @@
         <v>67</v>
       </c>
       <c r="G410">
-        <v>0.6793</v>
+        <v>0.6808</v>
       </c>
       <c r="H410">
-        <v>0.5164</v>
+        <v>0.5415</v>
       </c>
       <c r="I410">
-        <v>0.5978</v>
+        <v>0.6112</v>
       </c>
       <c r="J410">
-        <v>0.3207</v>
+        <v>0.3192</v>
       </c>
       <c r="K410">
-        <v>0.4836</v>
+        <v>0.4585</v>
       </c>
       <c r="L410">
-        <v>0.4022</v>
+        <v>0.3888</v>
       </c>
       <c r="M410">
         <v>179</v>
@@ -18659,22 +18659,22 @@
         <v>68</v>
       </c>
       <c r="G411">
-        <v>0.8529</v>
+        <v>0.8547</v>
       </c>
       <c r="H411">
         <v>0.7349</v>
       </c>
       <c r="I411">
-        <v>0.7939000000000001</v>
+        <v>0.7948</v>
       </c>
       <c r="J411">
-        <v>0.1471</v>
+        <v>0.1453</v>
       </c>
       <c r="K411">
         <v>0.2651</v>
       </c>
       <c r="L411">
-        <v>0.2061</v>
+        <v>0.2052</v>
       </c>
       <c r="M411">
         <v>179</v>
@@ -18838,19 +18838,19 @@
         <v>0.6859</v>
       </c>
       <c r="H415">
-        <v>0.4838</v>
+        <v>0.4796</v>
       </c>
       <c r="I415">
-        <v>0.5848</v>
+        <v>0.5828</v>
       </c>
       <c r="J415">
         <v>0.3141</v>
       </c>
       <c r="K415">
-        <v>0.5162</v>
+        <v>0.5204</v>
       </c>
       <c r="L415">
-        <v>0.4152</v>
+        <v>0.4172</v>
       </c>
       <c r="M415">
         <v>179</v>
@@ -18879,22 +18879,22 @@
         <v>67</v>
       </c>
       <c r="G416">
-        <v>0.6423</v>
+        <v>0.6454</v>
       </c>
       <c r="H416">
-        <v>0.4584</v>
+        <v>0.464</v>
       </c>
       <c r="I416">
-        <v>0.5504</v>
+        <v>0.5547</v>
       </c>
       <c r="J416">
-        <v>0.3577</v>
+        <v>0.3546</v>
       </c>
       <c r="K416">
-        <v>0.5416</v>
+        <v>0.536</v>
       </c>
       <c r="L416">
-        <v>0.4496</v>
+        <v>0.4453</v>
       </c>
       <c r="M416">
         <v>179</v>
@@ -19143,22 +19143,22 @@
         <v>68</v>
       </c>
       <c r="G422">
-        <v>0.853</v>
+        <v>0.8492</v>
       </c>
       <c r="H422">
-        <v>0.6915</v>
+        <v>0.6869</v>
       </c>
       <c r="I422">
-        <v>0.7722</v>
+        <v>0.768</v>
       </c>
       <c r="J422">
-        <v>0.147</v>
+        <v>0.1508</v>
       </c>
       <c r="K422">
-        <v>0.3085</v>
+        <v>0.3131</v>
       </c>
       <c r="L422">
-        <v>0.2278</v>
+        <v>0.232</v>
       </c>
       <c r="M422">
         <v>179</v>
@@ -19187,22 +19187,22 @@
         <v>69</v>
       </c>
       <c r="G423">
-        <v>0.8605</v>
+        <v>0.854</v>
       </c>
       <c r="H423">
-        <v>0.7062</v>
+        <v>0.7022</v>
       </c>
       <c r="I423">
-        <v>0.7834</v>
+        <v>0.7781</v>
       </c>
       <c r="J423">
-        <v>0.1395</v>
+        <v>0.146</v>
       </c>
       <c r="K423">
-        <v>0.2938</v>
+        <v>0.2978</v>
       </c>
       <c r="L423">
-        <v>0.2166</v>
+        <v>0.2219</v>
       </c>
       <c r="M423">
         <v>179</v>
@@ -19231,22 +19231,22 @@
         <v>70</v>
       </c>
       <c r="G424">
-        <v>0.8637</v>
+        <v>0.8613</v>
       </c>
       <c r="H424">
-        <v>0.7413</v>
+        <v>0.7388</v>
       </c>
       <c r="I424">
-        <v>0.8025</v>
+        <v>0.8</v>
       </c>
       <c r="J424">
-        <v>0.1363</v>
+        <v>0.1387</v>
       </c>
       <c r="K424">
-        <v>0.2587</v>
+        <v>0.2612</v>
       </c>
       <c r="L424">
-        <v>0.1975</v>
+        <v>0.2</v>
       </c>
       <c r="M424">
         <v>179</v>
@@ -19275,22 +19275,22 @@
         <v>71</v>
       </c>
       <c r="G425">
-        <v>0.4478</v>
+        <v>0.441</v>
       </c>
       <c r="H425">
-        <v>0.3556</v>
+        <v>0.3473</v>
       </c>
       <c r="I425">
-        <v>0.4017</v>
+        <v>0.3942</v>
       </c>
       <c r="J425">
-        <v>0.5522</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="K425">
-        <v>0.6444</v>
+        <v>0.6526999999999999</v>
       </c>
       <c r="L425">
-        <v>0.5983000000000001</v>
+        <v>0.6058</v>
       </c>
       <c r="M425">
         <v>179</v>
@@ -19319,22 +19319,22 @@
         <v>73</v>
       </c>
       <c r="G426">
-        <v>0.5644</v>
+        <v>0.5464</v>
       </c>
       <c r="H426">
-        <v>0.4298</v>
+        <v>0.4207</v>
       </c>
       <c r="I426">
-        <v>0.4971</v>
+        <v>0.4836</v>
       </c>
       <c r="J426">
-        <v>0.4356</v>
+        <v>0.4536</v>
       </c>
       <c r="K426">
-        <v>0.5702</v>
+        <v>0.5793</v>
       </c>
       <c r="L426">
-        <v>0.5029</v>
+        <v>0.5164</v>
       </c>
       <c r="M426">
         <v>179</v>
@@ -19498,19 +19498,19 @@
         <v>0.2788</v>
       </c>
       <c r="H430">
-        <v>0.1517</v>
+        <v>0.1507</v>
       </c>
       <c r="I430">
-        <v>0.2152</v>
+        <v>0.2148</v>
       </c>
       <c r="J430">
         <v>0.7212</v>
       </c>
       <c r="K430">
-        <v>0.8483000000000001</v>
+        <v>0.8493000000000001</v>
       </c>
       <c r="L430">
-        <v>0.7848000000000001</v>
+        <v>0.7852</v>
       </c>
       <c r="M430">
         <v>179</v>
@@ -19627,22 +19627,22 @@
         <v>73</v>
       </c>
       <c r="G433">
-        <v>0.2775</v>
+        <v>0.2736</v>
       </c>
       <c r="H433">
         <v>0.1373</v>
       </c>
       <c r="I433">
-        <v>0.2074</v>
+        <v>0.2054</v>
       </c>
       <c r="J433">
-        <v>0.7225</v>
+        <v>0.7264</v>
       </c>
       <c r="K433">
         <v>0.8627</v>
       </c>
       <c r="L433">
-        <v>0.7926</v>
+        <v>0.7946</v>
       </c>
       <c r="M433">
         <v>179</v>
@@ -19674,19 +19674,19 @@
         <v>0.2526</v>
       </c>
       <c r="H434">
-        <v>0.1328</v>
+        <v>0.1302</v>
       </c>
       <c r="I434">
-        <v>0.1927</v>
+        <v>0.1914</v>
       </c>
       <c r="J434">
         <v>0.7474</v>
       </c>
       <c r="K434">
-        <v>0.8672</v>
+        <v>0.8698</v>
       </c>
       <c r="L434">
-        <v>0.8073</v>
+        <v>0.8086</v>
       </c>
       <c r="M434">
         <v>179</v>
@@ -19715,22 +19715,22 @@
         <v>73</v>
       </c>
       <c r="G435">
-        <v>0.2435</v>
+        <v>0.2411</v>
       </c>
       <c r="H435">
-        <v>0.1407</v>
+        <v>0.1383</v>
       </c>
       <c r="I435">
-        <v>0.1921</v>
+        <v>0.1897</v>
       </c>
       <c r="J435">
-        <v>0.7565</v>
+        <v>0.7589</v>
       </c>
       <c r="K435">
-        <v>0.8593</v>
+        <v>0.8617</v>
       </c>
       <c r="L435">
-        <v>0.8079</v>
+        <v>0.8103</v>
       </c>
       <c r="M435">
         <v>179</v>
@@ -19762,19 +19762,19 @@
         <v>0.6656</v>
       </c>
       <c r="H436">
-        <v>0.5263</v>
+        <v>0.5189</v>
       </c>
       <c r="I436">
-        <v>0.596</v>
+        <v>0.5921999999999999</v>
       </c>
       <c r="J436">
         <v>0.3344</v>
       </c>
       <c r="K436">
-        <v>0.4737</v>
+        <v>0.4811</v>
       </c>
       <c r="L436">
-        <v>0.404</v>
+        <v>0.4078</v>
       </c>
       <c r="M436">
         <v>179</v>

</xml_diff>